<commit_message>
Mark the Pole Star on easier settings; plan: R1 watching, F33 in progress after first playtest
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018inbrQHz2eFfbj9ny1keZA
</commit_message>
<xml_diff>
--- a/docs/Vinland_Game_Development_Plan.xlsx
+++ b/docs/Vinland_Game_Development_Plan.xlsx
@@ -86,7 +86,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1890" uniqueCount="1166">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1890" uniqueCount="1167">
   <si>
     <t xml:space="preserve">VINLAND</t>
   </si>
@@ -2479,7 +2479,7 @@
     <t xml:space="preserve">Polish</t>
   </si>
   <si>
-    <t xml:space="preserve">Forgiveness tuned from playtest 2 logs.</t>
+    <t xml:space="preserve">Forgiveness tuned from playtest 2 logs.  [Difficulty levels and novice-player tests in place from the first playtest; tune again from real play logs.]</t>
   </si>
   <si>
     <t xml:space="preserve">F56</t>
@@ -2956,25 +2956,28 @@
     <t xml:space="preserve">Star ring is not fun</t>
   </si>
   <si>
-    <t xml:space="preserve">Stop at the slice. Retune forgiveness before any other verb.</t>
+    <t xml:space="preserve">Stop at the slice. Retune forgiveness before any other verb. [17 Oct 2026: first playtest failed every mini-game. Retuned: Forgiving / Standard / Hard difficulty, guided prompts, keyboard wind-up, novice-player bots now gate every build.]</t>
   </si>
   <si>
     <t xml:space="preserve">Table testers stop seating stars after three tries</t>
   </si>
   <si>
+    <t xml:space="preserve">Watching</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hold math is trivial or cruel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Log every slice run. Tune food coverage on Assumptions, not in code literals.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Slice runs end with the hold always full or never touched</t>
+  </si>
+  <si>
     <t xml:space="preserve">Open</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hold math is trivial or cruel</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Log every slice run. Tune food coverage on Assumptions, not in code literals.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Slice runs end with the hold always full or never touched</t>
   </si>
   <si>
     <t xml:space="preserve">R3</t>
@@ -4788,11 +4791,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="73134574"/>
-        <c:axId val="63984756"/>
+        <c:axId val="98654844"/>
+        <c:axId val="96776336"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="73134574"/>
+        <c:axId val="98654844"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4824,7 +4827,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="63984756"/>
+        <c:crossAx val="96776336"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -4832,7 +4835,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="63984756"/>
+        <c:axId val="96776336"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4908,7 +4911,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="73134574"/>
+        <c:crossAx val="98654844"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -4947,9 +4950,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>744120</xdr:colOff>
+      <xdr:colOff>743760</xdr:colOff>
       <xdr:row>40</xdr:row>
-      <xdr:rowOff>60480</xdr:rowOff>
+      <xdr:rowOff>60120</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -4958,7 +4961,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="0" y="6562800"/>
-        <a:ext cx="5396040" cy="2156040"/>
+        <a:ext cx="5395680" cy="2155680"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -7745,15 +7748,15 @@
         <v>962</v>
       </c>
       <c r="J6" s="69" t="s">
-        <v>958</v>
+        <v>963</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="58" t="s">
-        <v>963</v>
+        <v>964</v>
       </c>
       <c r="B7" s="58" t="s">
-        <v>964</v>
+        <v>965</v>
       </c>
       <c r="C7" s="43" t="n">
         <v>2</v>
@@ -7766,7 +7769,7 @@
         <v>8</v>
       </c>
       <c r="F7" s="58" t="s">
-        <v>965</v>
+        <v>966</v>
       </c>
       <c r="G7" s="58" t="s">
         <v>631</v>
@@ -7775,18 +7778,18 @@
         <v>855</v>
       </c>
       <c r="I7" s="58" t="s">
-        <v>966</v>
+        <v>967</v>
       </c>
       <c r="J7" s="69" t="s">
-        <v>958</v>
+        <v>963</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="58" t="s">
-        <v>967</v>
+        <v>968</v>
       </c>
       <c r="B8" s="58" t="s">
-        <v>968</v>
+        <v>969</v>
       </c>
       <c r="C8" s="43" t="n">
         <v>4</v>
@@ -7799,7 +7802,7 @@
         <v>12</v>
       </c>
       <c r="F8" s="58" t="s">
-        <v>969</v>
+        <v>970</v>
       </c>
       <c r="G8" s="58" t="s">
         <v>100</v>
@@ -7808,18 +7811,18 @@
         <v>847</v>
       </c>
       <c r="I8" s="58" t="s">
-        <v>970</v>
+        <v>971</v>
       </c>
       <c r="J8" s="69" t="s">
-        <v>958</v>
+        <v>963</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="58" t="s">
-        <v>971</v>
+        <v>972</v>
       </c>
       <c r="B9" s="58" t="s">
-        <v>972</v>
+        <v>973</v>
       </c>
       <c r="C9" s="43" t="n">
         <v>2</v>
@@ -7832,7 +7835,7 @@
         <v>6</v>
       </c>
       <c r="F9" s="58" t="s">
-        <v>973</v>
+        <v>974</v>
       </c>
       <c r="G9" s="58" t="s">
         <v>639</v>
@@ -7841,18 +7844,18 @@
         <v>847</v>
       </c>
       <c r="I9" s="58" t="s">
-        <v>974</v>
+        <v>975</v>
       </c>
       <c r="J9" s="69" t="s">
-        <v>958</v>
+        <v>963</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="58" t="s">
-        <v>975</v>
+        <v>976</v>
       </c>
       <c r="B10" s="58" t="s">
-        <v>976</v>
+        <v>977</v>
       </c>
       <c r="C10" s="43" t="n">
         <v>2</v>
@@ -7865,7 +7868,7 @@
         <v>10</v>
       </c>
       <c r="F10" s="58" t="s">
-        <v>977</v>
+        <v>978</v>
       </c>
       <c r="G10" s="58" t="s">
         <v>292</v>
@@ -7874,18 +7877,18 @@
         <v>847</v>
       </c>
       <c r="I10" s="58" t="s">
-        <v>978</v>
+        <v>979</v>
       </c>
       <c r="J10" s="69" t="s">
-        <v>958</v>
+        <v>963</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="58" t="s">
-        <v>979</v>
+        <v>980</v>
       </c>
       <c r="B11" s="58" t="s">
-        <v>980</v>
+        <v>981</v>
       </c>
       <c r="C11" s="43" t="n">
         <v>3</v>
@@ -7898,7 +7901,7 @@
         <v>12</v>
       </c>
       <c r="F11" s="58" t="s">
-        <v>981</v>
+        <v>982</v>
       </c>
       <c r="G11" s="58" t="s">
         <v>100</v>
@@ -7907,18 +7910,18 @@
         <v>851</v>
       </c>
       <c r="I11" s="58" t="s">
-        <v>982</v>
+        <v>983</v>
       </c>
       <c r="J11" s="69" t="s">
-        <v>958</v>
+        <v>963</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="58" t="s">
-        <v>983</v>
+        <v>984</v>
       </c>
       <c r="B12" s="58" t="s">
-        <v>984</v>
+        <v>985</v>
       </c>
       <c r="C12" s="43" t="n">
         <v>2</v>
@@ -7931,7 +7934,7 @@
         <v>8</v>
       </c>
       <c r="F12" s="58" t="s">
-        <v>985</v>
+        <v>986</v>
       </c>
       <c r="G12" s="58" t="s">
         <v>631</v>
@@ -7940,18 +7943,18 @@
         <v>839</v>
       </c>
       <c r="I12" s="58" t="s">
-        <v>986</v>
+        <v>987</v>
       </c>
       <c r="J12" s="69" t="s">
-        <v>958</v>
+        <v>963</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="58" t="s">
-        <v>987</v>
+        <v>988</v>
       </c>
       <c r="B13" s="58" t="s">
-        <v>988</v>
+        <v>989</v>
       </c>
       <c r="C13" s="43" t="n">
         <v>2</v>
@@ -7964,7 +7967,7 @@
         <v>4</v>
       </c>
       <c r="F13" s="58" t="s">
-        <v>989</v>
+        <v>990</v>
       </c>
       <c r="G13" s="58" t="s">
         <v>292</v>
@@ -7973,18 +7976,18 @@
         <v>839</v>
       </c>
       <c r="I13" s="58" t="s">
-        <v>990</v>
+        <v>991</v>
       </c>
       <c r="J13" s="69" t="s">
-        <v>958</v>
+        <v>963</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="58" t="s">
-        <v>991</v>
+        <v>992</v>
       </c>
       <c r="B14" s="58" t="s">
-        <v>992</v>
+        <v>993</v>
       </c>
       <c r="C14" s="43" t="n">
         <v>3</v>
@@ -7997,7 +8000,7 @@
         <v>12</v>
       </c>
       <c r="F14" s="58" t="s">
-        <v>993</v>
+        <v>994</v>
       </c>
       <c r="G14" s="58" t="s">
         <v>292</v>
@@ -8006,18 +8009,18 @@
         <v>851</v>
       </c>
       <c r="I14" s="58" t="s">
-        <v>994</v>
+        <v>995</v>
       </c>
       <c r="J14" s="69" t="s">
-        <v>958</v>
+        <v>963</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="58" t="s">
-        <v>995</v>
+        <v>996</v>
       </c>
       <c r="B15" s="58" t="s">
-        <v>996</v>
+        <v>997</v>
       </c>
       <c r="C15" s="43" t="n">
         <v>3</v>
@@ -8030,7 +8033,7 @@
         <v>15</v>
       </c>
       <c r="F15" s="58" t="s">
-        <v>997</v>
+        <v>998</v>
       </c>
       <c r="G15" s="58" t="s">
         <v>292</v>
@@ -8039,18 +8042,18 @@
         <v>847</v>
       </c>
       <c r="I15" s="58" t="s">
-        <v>998</v>
+        <v>999</v>
       </c>
       <c r="J15" s="69" t="s">
-        <v>958</v>
+        <v>963</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="58" t="s">
-        <v>999</v>
+        <v>1000</v>
       </c>
       <c r="B16" s="58" t="s">
-        <v>1000</v>
+        <v>1001</v>
       </c>
       <c r="C16" s="43" t="n">
         <v>4</v>
@@ -8063,7 +8066,7 @@
         <v>16</v>
       </c>
       <c r="F16" s="58" t="s">
-        <v>1001</v>
+        <v>1002</v>
       </c>
       <c r="G16" s="58" t="s">
         <v>100</v>
@@ -8072,18 +8075,18 @@
         <v>843</v>
       </c>
       <c r="I16" s="58" t="s">
-        <v>1002</v>
+        <v>1003</v>
       </c>
       <c r="J16" s="69" t="s">
-        <v>958</v>
+        <v>963</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="58" t="s">
-        <v>1003</v>
+        <v>1004</v>
       </c>
       <c r="B17" s="58" t="s">
-        <v>1004</v>
+        <v>1005</v>
       </c>
       <c r="C17" s="43" t="n">
         <v>3</v>
@@ -8096,7 +8099,7 @@
         <v>12</v>
       </c>
       <c r="F17" s="58" t="s">
-        <v>1005</v>
+        <v>1006</v>
       </c>
       <c r="G17" s="58" t="s">
         <v>100</v>
@@ -8105,18 +8108,18 @@
         <v>847</v>
       </c>
       <c r="I17" s="58" t="s">
-        <v>1006</v>
+        <v>1007</v>
       </c>
       <c r="J17" s="69" t="s">
-        <v>958</v>
+        <v>963</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="58" t="s">
-        <v>1007</v>
+        <v>1008</v>
       </c>
       <c r="B18" s="58" t="s">
-        <v>1008</v>
+        <v>1009</v>
       </c>
       <c r="C18" s="43" t="n">
         <v>2</v>
@@ -8129,7 +8132,7 @@
         <v>6</v>
       </c>
       <c r="F18" s="58" t="s">
-        <v>1009</v>
+        <v>1010</v>
       </c>
       <c r="G18" s="58" t="s">
         <v>292</v>
@@ -8138,18 +8141,18 @@
         <v>855</v>
       </c>
       <c r="I18" s="58" t="s">
-        <v>1010</v>
+        <v>1011</v>
       </c>
       <c r="J18" s="69" t="s">
-        <v>958</v>
+        <v>963</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="58" t="s">
-        <v>1011</v>
+        <v>1012</v>
       </c>
       <c r="B19" s="58" t="s">
-        <v>1012</v>
+        <v>1013</v>
       </c>
       <c r="C19" s="43" t="n">
         <v>2</v>
@@ -8162,7 +8165,7 @@
         <v>8</v>
       </c>
       <c r="F19" s="58" t="s">
-        <v>1013</v>
+        <v>1014</v>
       </c>
       <c r="G19" s="58" t="s">
         <v>631</v>
@@ -8171,18 +8174,18 @@
         <v>847</v>
       </c>
       <c r="I19" s="58" t="s">
-        <v>1014</v>
+        <v>1015</v>
       </c>
       <c r="J19" s="69" t="s">
-        <v>958</v>
+        <v>963</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="58" t="s">
-        <v>1015</v>
+        <v>1016</v>
       </c>
       <c r="B20" s="58" t="s">
-        <v>1016</v>
+        <v>1017</v>
       </c>
       <c r="C20" s="43" t="n">
         <v>3</v>
@@ -8195,7 +8198,7 @@
         <v>15</v>
       </c>
       <c r="F20" s="58" t="s">
-        <v>1017</v>
+        <v>1018</v>
       </c>
       <c r="G20" s="58" t="s">
         <v>100</v>
@@ -8204,10 +8207,10 @@
         <v>843</v>
       </c>
       <c r="I20" s="58" t="s">
-        <v>1018</v>
+        <v>1019</v>
       </c>
       <c r="J20" s="69" t="s">
-        <v>958</v>
+        <v>963</v>
       </c>
     </row>
   </sheetData>
@@ -8285,7 +8288,7 @@
     </row>
     <row r="2" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>1019</v>
+        <v>1020</v>
       </c>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
@@ -8296,16 +8299,16 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="57" t="s">
-        <v>1020</v>
+        <v>1021</v>
       </c>
       <c r="B4" s="57" t="s">
-        <v>1021</v>
+        <v>1022</v>
       </c>
       <c r="C4" s="57" t="s">
-        <v>1022</v>
+        <v>1023</v>
       </c>
       <c r="D4" s="57" t="s">
-        <v>1023</v>
+        <v>1024</v>
       </c>
       <c r="E4" s="57" t="s">
         <v>95</v>
@@ -8314,30 +8317,30 @@
         <v>619</v>
       </c>
       <c r="G4" s="9" t="s">
-        <v>1024</v>
+        <v>1025</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="27" t="s">
-        <v>1025</v>
+        <v>1026</v>
       </c>
       <c r="B5" s="27" t="s">
-        <v>1026</v>
+        <v>1027</v>
       </c>
       <c r="C5" s="27" t="s">
-        <v>1027</v>
+        <v>1028</v>
       </c>
       <c r="D5" s="27" t="s">
-        <v>1028</v>
+        <v>1029</v>
       </c>
       <c r="E5" s="27" t="s">
-        <v>1029</v>
+        <v>1030</v>
       </c>
       <c r="F5" s="27" t="s">
         <v>639</v>
       </c>
       <c r="G5" s="27" t="s">
-        <v>1030</v>
+        <v>1031</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8345,68 +8348,68 @@
         <v>591</v>
       </c>
       <c r="B6" s="58" t="s">
-        <v>1031</v>
+        <v>1032</v>
       </c>
       <c r="C6" s="58" t="s">
-        <v>1032</v>
+        <v>1033</v>
       </c>
       <c r="D6" s="58" t="s">
-        <v>1033</v>
+        <v>1034</v>
       </c>
       <c r="E6" s="58" t="s">
-        <v>1034</v>
+        <v>1035</v>
       </c>
       <c r="F6" s="58" t="s">
-        <v>1035</v>
+        <v>1036</v>
       </c>
       <c r="G6" s="58" t="s">
-        <v>1036</v>
+        <v>1037</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="27" t="s">
-        <v>1037</v>
+        <v>1038</v>
       </c>
       <c r="B7" s="27" t="s">
-        <v>1038</v>
+        <v>1039</v>
       </c>
       <c r="C7" s="27" t="s">
-        <v>1039</v>
+        <v>1040</v>
       </c>
       <c r="D7" s="27" t="s">
-        <v>1040</v>
+        <v>1041</v>
       </c>
       <c r="E7" s="27" t="s">
-        <v>1041</v>
+        <v>1042</v>
       </c>
       <c r="F7" s="27" t="s">
         <v>639</v>
       </c>
       <c r="G7" s="27" t="s">
-        <v>1036</v>
+        <v>1037</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="58" t="s">
-        <v>1042</v>
+        <v>1043</v>
       </c>
       <c r="B8" s="58" t="s">
-        <v>1043</v>
+        <v>1044</v>
       </c>
       <c r="C8" s="58" t="s">
-        <v>1044</v>
+        <v>1045</v>
       </c>
       <c r="D8" s="58" t="s">
-        <v>1045</v>
+        <v>1046</v>
       </c>
       <c r="E8" s="58" t="s">
-        <v>1046</v>
+        <v>1047</v>
       </c>
       <c r="F8" s="58" t="s">
         <v>639</v>
       </c>
       <c r="G8" s="58" t="s">
-        <v>1047</v>
+        <v>1048</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8414,22 +8417,22 @@
         <v>476</v>
       </c>
       <c r="B9" s="27" t="s">
-        <v>1048</v>
+        <v>1049</v>
       </c>
       <c r="C9" s="27" t="s">
-        <v>1049</v>
+        <v>1050</v>
       </c>
       <c r="D9" s="27" t="s">
-        <v>1050</v>
+        <v>1051</v>
       </c>
       <c r="E9" s="27" t="s">
-        <v>1051</v>
+        <v>1052</v>
       </c>
       <c r="F9" s="27" t="s">
         <v>639</v>
       </c>
       <c r="G9" s="27" t="s">
-        <v>1052</v>
+        <v>1053</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8437,22 +8440,22 @@
         <v>667</v>
       </c>
       <c r="B10" s="58" t="s">
-        <v>1053</v>
+        <v>1054</v>
       </c>
       <c r="C10" s="58" t="s">
-        <v>1054</v>
+        <v>1055</v>
       </c>
       <c r="D10" s="58" t="s">
         <v>789</v>
       </c>
       <c r="E10" s="58" t="s">
-        <v>1055</v>
+        <v>1056</v>
       </c>
       <c r="F10" s="58" t="s">
         <v>639</v>
       </c>
       <c r="G10" s="58" t="s">
-        <v>1056</v>
+        <v>1057</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8460,22 +8463,22 @@
         <v>731</v>
       </c>
       <c r="B11" s="27" t="s">
-        <v>1057</v>
+        <v>1058</v>
       </c>
       <c r="C11" s="27" t="s">
-        <v>1058</v>
+        <v>1059</v>
       </c>
       <c r="D11" s="27" t="s">
-        <v>1059</v>
+        <v>1060</v>
       </c>
       <c r="E11" s="27" t="s">
-        <v>1060</v>
+        <v>1061</v>
       </c>
       <c r="F11" s="27" t="s">
         <v>731</v>
       </c>
       <c r="G11" s="27" t="s">
-        <v>1061</v>
+        <v>1062</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8483,91 +8486,91 @@
         <v>750</v>
       </c>
       <c r="B12" s="58" t="s">
-        <v>1062</v>
+        <v>1063</v>
       </c>
       <c r="C12" s="58" t="s">
-        <v>1063</v>
+        <v>1064</v>
       </c>
       <c r="D12" s="58" t="s">
-        <v>1064</v>
+        <v>1065</v>
       </c>
       <c r="E12" s="58" t="s">
-        <v>1065</v>
+        <v>1066</v>
       </c>
       <c r="F12" s="58" t="s">
         <v>292</v>
       </c>
       <c r="G12" s="58" t="s">
-        <v>1036</v>
+        <v>1037</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="27" t="s">
-        <v>1066</v>
+        <v>1067</v>
       </c>
       <c r="B13" s="27" t="s">
-        <v>1067</v>
+        <v>1068</v>
       </c>
       <c r="C13" s="27" t="s">
-        <v>1068</v>
+        <v>1069</v>
       </c>
       <c r="D13" s="27" t="s">
-        <v>1069</v>
+        <v>1070</v>
       </c>
       <c r="E13" s="27" t="s">
-        <v>1070</v>
+        <v>1071</v>
       </c>
       <c r="F13" s="27" t="s">
         <v>631</v>
       </c>
       <c r="G13" s="27" t="s">
-        <v>1036</v>
+        <v>1037</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="58" t="s">
-        <v>1071</v>
+        <v>1072</v>
       </c>
       <c r="B14" s="58" t="s">
-        <v>1072</v>
+        <v>1073</v>
       </c>
       <c r="C14" s="58" t="s">
-        <v>1073</v>
+        <v>1074</v>
       </c>
       <c r="D14" s="58" t="s">
-        <v>1074</v>
+        <v>1075</v>
       </c>
       <c r="E14" s="58" t="s">
-        <v>1075</v>
+        <v>1076</v>
       </c>
       <c r="F14" s="58" t="s">
         <v>100</v>
       </c>
       <c r="G14" s="58" t="s">
-        <v>1076</v>
+        <v>1077</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="27" t="s">
-        <v>1077</v>
+        <v>1078</v>
       </c>
       <c r="B15" s="27" t="s">
-        <v>1078</v>
+        <v>1079</v>
       </c>
       <c r="C15" s="27" t="s">
-        <v>1079</v>
+        <v>1080</v>
       </c>
       <c r="D15" s="27" t="s">
-        <v>1080</v>
+        <v>1081</v>
       </c>
       <c r="E15" s="27" t="s">
-        <v>1081</v>
+        <v>1082</v>
       </c>
       <c r="F15" s="27" t="s">
         <v>100</v>
       </c>
       <c r="G15" s="27" t="s">
-        <v>1082</v>
+        <v>1083</v>
       </c>
     </row>
   </sheetData>
@@ -8609,7 +8612,7 @@
     </row>
     <row r="2" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>1083</v>
+        <v>1084</v>
       </c>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
@@ -8620,10 +8623,10 @@
         <v>110</v>
       </c>
       <c r="B4" s="57" t="s">
-        <v>1084</v>
+        <v>1085</v>
       </c>
       <c r="C4" s="57" t="s">
-        <v>1085</v>
+        <v>1086</v>
       </c>
       <c r="D4" s="57" t="s">
         <v>619</v>
@@ -8631,10 +8634,10 @@
     </row>
     <row r="5" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="27" t="s">
-        <v>1086</v>
+        <v>1087</v>
       </c>
       <c r="B5" s="27" t="s">
-        <v>1087</v>
+        <v>1088</v>
       </c>
       <c r="C5" s="27" t="s">
         <v>839</v>
@@ -8645,13 +8648,13 @@
     </row>
     <row r="6" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="58" t="s">
-        <v>1088</v>
+        <v>1089</v>
       </c>
       <c r="B6" s="58" t="s">
-        <v>1089</v>
+        <v>1090</v>
       </c>
       <c r="C6" s="58" t="s">
-        <v>1090</v>
+        <v>1091</v>
       </c>
       <c r="D6" s="58" t="s">
         <v>631</v>
@@ -8659,10 +8662,10 @@
     </row>
     <row r="7" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="27" t="s">
-        <v>1091</v>
+        <v>1092</v>
       </c>
       <c r="B7" s="27" t="s">
-        <v>1092</v>
+        <v>1093</v>
       </c>
       <c r="C7" s="27" t="s">
         <v>847</v>
@@ -8673,10 +8676,10 @@
     </row>
     <row r="8" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="58" t="s">
-        <v>1093</v>
+        <v>1094</v>
       </c>
       <c r="B8" s="58" t="s">
-        <v>1094</v>
+        <v>1095</v>
       </c>
       <c r="C8" s="58" t="s">
         <v>843</v>
@@ -8687,10 +8690,10 @@
     </row>
     <row r="9" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="27" t="s">
-        <v>1095</v>
+        <v>1096</v>
       </c>
       <c r="B9" s="27" t="s">
-        <v>1096</v>
+        <v>1097</v>
       </c>
       <c r="C9" s="27" t="s">
         <v>839</v>
@@ -8701,10 +8704,10 @@
     </row>
     <row r="10" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="58" t="s">
-        <v>1097</v>
+        <v>1098</v>
       </c>
       <c r="B10" s="58" t="s">
-        <v>1098</v>
+        <v>1099</v>
       </c>
       <c r="C10" s="58" t="s">
         <v>847</v>
@@ -8715,10 +8718,10 @@
     </row>
     <row r="11" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="27" t="s">
-        <v>1099</v>
+        <v>1100</v>
       </c>
       <c r="B11" s="27" t="s">
-        <v>1100</v>
+        <v>1101</v>
       </c>
       <c r="C11" s="27" t="s">
         <v>855</v>
@@ -8729,10 +8732,10 @@
     </row>
     <row r="12" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="58" t="s">
-        <v>1101</v>
+        <v>1102</v>
       </c>
       <c r="B12" s="58" t="s">
-        <v>1102</v>
+        <v>1103</v>
       </c>
       <c r="C12" s="58" t="s">
         <v>858</v>
@@ -8743,10 +8746,10 @@
     </row>
     <row r="13" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="27" t="s">
-        <v>1103</v>
+        <v>1104</v>
       </c>
       <c r="B13" s="27" t="s">
-        <v>1104</v>
+        <v>1105</v>
       </c>
       <c r="C13" s="27" t="s">
         <v>858</v>
@@ -8757,13 +8760,13 @@
     </row>
     <row r="14" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="58" t="s">
-        <v>1105</v>
+        <v>1106</v>
       </c>
       <c r="B14" s="58" t="s">
-        <v>1106</v>
+        <v>1107</v>
       </c>
       <c r="C14" s="58" t="s">
-        <v>1107</v>
+        <v>1108</v>
       </c>
       <c r="D14" s="58" t="s">
         <v>292</v>
@@ -8771,10 +8774,10 @@
     </row>
     <row r="15" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="27" t="s">
-        <v>1108</v>
+        <v>1109</v>
       </c>
       <c r="B15" s="27" t="s">
-        <v>1109</v>
+        <v>1110</v>
       </c>
       <c r="C15" s="27" t="s">
         <v>843</v>
@@ -8785,7 +8788,7 @@
     </row>
     <row r="16" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="58" t="s">
-        <v>1110</v>
+        <v>1111</v>
       </c>
       <c r="B16" s="58" t="str">
         <f aca="false">"Premium at $"&amp;TEXT(Assumptions!B69,"0.00")&amp;". Launch discount no deeper than the realized-price factor on Assumptions."</f>
@@ -8800,10 +8803,10 @@
     </row>
     <row r="17" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="27" t="s">
-        <v>1111</v>
+        <v>1112</v>
       </c>
       <c r="B17" s="27" t="s">
-        <v>1112</v>
+        <v>1113</v>
       </c>
       <c r="C17" s="27" t="s">
         <v>843</v>
@@ -8817,7 +8820,7 @@
         <v>833</v>
       </c>
       <c r="B18" s="58" t="s">
-        <v>1113</v>
+        <v>1114</v>
       </c>
       <c r="C18" s="58" t="s">
         <v>851</v>
@@ -8828,10 +8831,10 @@
     </row>
     <row r="19" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="27" t="s">
-        <v>1114</v>
+        <v>1115</v>
       </c>
       <c r="B19" s="27" t="s">
-        <v>1115</v>
+        <v>1116</v>
       </c>
       <c r="C19" s="27" t="s">
         <v>855</v>
@@ -8842,10 +8845,10 @@
     </row>
     <row r="20" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="58" t="s">
-        <v>1116</v>
+        <v>1117</v>
       </c>
       <c r="B20" s="58" t="s">
-        <v>1117</v>
+        <v>1118</v>
       </c>
       <c r="C20" s="58" t="s">
         <v>855</v>
@@ -8856,10 +8859,10 @@
     </row>
     <row r="21" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="27" t="s">
-        <v>1118</v>
+        <v>1119</v>
       </c>
       <c r="B21" s="27" t="s">
-        <v>1119</v>
+        <v>1120</v>
       </c>
       <c r="C21" s="27" t="s">
         <v>855</v>
@@ -8870,10 +8873,10 @@
     </row>
     <row r="22" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="58" t="s">
-        <v>1120</v>
+        <v>1121</v>
       </c>
       <c r="B22" s="58" t="s">
-        <v>1121</v>
+        <v>1122</v>
       </c>
       <c r="C22" s="58" t="s">
         <v>858</v>
@@ -8922,7 +8925,7 @@
     </row>
     <row r="2" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>1122</v>
+        <v>1123</v>
       </c>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
@@ -8930,16 +8933,16 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>1123</v>
+        <v>1124</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>1124</v>
+        <v>1125</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>1125</v>
+        <v>1126</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>1126</v>
+        <v>1127</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8947,13 +8950,13 @@
         <v>46311</v>
       </c>
       <c r="B5" s="27" t="s">
-        <v>1127</v>
+        <v>1128</v>
       </c>
       <c r="C5" s="27" t="s">
-        <v>1128</v>
+        <v>1129</v>
       </c>
       <c r="D5" s="27" t="s">
-        <v>1129</v>
+        <v>1130</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8961,13 +8964,13 @@
         <v>46311</v>
       </c>
       <c r="B6" s="58" t="s">
-        <v>1127</v>
+        <v>1128</v>
       </c>
       <c r="C6" s="58" t="s">
-        <v>1130</v>
+        <v>1131</v>
       </c>
       <c r="D6" s="58" t="s">
-        <v>1131</v>
+        <v>1132</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8975,13 +8978,13 @@
         <v>46311</v>
       </c>
       <c r="B7" s="27" t="s">
-        <v>1127</v>
+        <v>1128</v>
       </c>
       <c r="C7" s="27" t="s">
-        <v>1132</v>
+        <v>1133</v>
       </c>
       <c r="D7" s="27" t="s">
-        <v>1133</v>
+        <v>1134</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8992,10 +8995,10 @@
         <v>893</v>
       </c>
       <c r="C8" s="58" t="s">
-        <v>1134</v>
+        <v>1135</v>
       </c>
       <c r="D8" s="58" t="s">
-        <v>1135</v>
+        <v>1136</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9003,13 +9006,13 @@
         <v>46311</v>
       </c>
       <c r="B9" s="27" t="s">
-        <v>1136</v>
+        <v>1137</v>
       </c>
       <c r="C9" s="27" t="s">
-        <v>1137</v>
+        <v>1138</v>
       </c>
       <c r="D9" s="27" t="s">
-        <v>1138</v>
+        <v>1139</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9020,10 +9023,10 @@
         <v>53</v>
       </c>
       <c r="C10" s="58" t="s">
-        <v>1139</v>
+        <v>1140</v>
       </c>
       <c r="D10" s="58" t="s">
-        <v>1140</v>
+        <v>1141</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9031,13 +9034,13 @@
         <v>46311</v>
       </c>
       <c r="B11" s="27" t="s">
-        <v>1141</v>
+        <v>1142</v>
       </c>
       <c r="C11" s="27" t="s">
-        <v>1142</v>
+        <v>1143</v>
       </c>
       <c r="D11" s="27" t="s">
-        <v>1143</v>
+        <v>1144</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9048,10 +9051,10 @@
         <v>372</v>
       </c>
       <c r="C12" s="58" t="s">
-        <v>1144</v>
+        <v>1145</v>
       </c>
       <c r="D12" s="58" t="s">
-        <v>1145</v>
+        <v>1146</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9059,13 +9062,13 @@
         <v>46311</v>
       </c>
       <c r="B13" s="27" t="s">
-        <v>1146</v>
+        <v>1147</v>
       </c>
       <c r="C13" s="27" t="s">
-        <v>1147</v>
+        <v>1148</v>
       </c>
       <c r="D13" s="27" t="s">
-        <v>1148</v>
+        <v>1149</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9073,13 +9076,13 @@
         <v>46311</v>
       </c>
       <c r="B14" s="58" t="s">
-        <v>1149</v>
+        <v>1150</v>
       </c>
       <c r="C14" s="58" t="s">
-        <v>1150</v>
+        <v>1151</v>
       </c>
       <c r="D14" s="58" t="s">
-        <v>1151</v>
+        <v>1152</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9090,10 +9093,10 @@
         <v>58</v>
       </c>
       <c r="C15" s="27" t="s">
-        <v>1152</v>
+        <v>1153</v>
       </c>
       <c r="D15" s="27" t="s">
-        <v>1153</v>
+        <v>1154</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9101,13 +9104,13 @@
         <v>46311</v>
       </c>
       <c r="B16" s="58" t="s">
-        <v>1154</v>
+        <v>1155</v>
       </c>
       <c r="C16" s="58" t="s">
-        <v>1155</v>
+        <v>1156</v>
       </c>
       <c r="D16" s="58" t="s">
-        <v>1156</v>
+        <v>1157</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9118,10 +9121,10 @@
         <v>62</v>
       </c>
       <c r="C17" s="27" t="s">
-        <v>1157</v>
+        <v>1158</v>
       </c>
       <c r="D17" s="27" t="s">
-        <v>1158</v>
+        <v>1159</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9132,10 +9135,10 @@
         <v>406</v>
       </c>
       <c r="C18" s="58" t="s">
-        <v>1159</v>
+        <v>1160</v>
       </c>
       <c r="D18" s="58" t="s">
-        <v>1160</v>
+        <v>1161</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9146,10 +9149,10 @@
         <v>682</v>
       </c>
       <c r="C19" s="27" t="s">
-        <v>1161</v>
+        <v>1162</v>
       </c>
       <c r="D19" s="27" t="s">
-        <v>1162</v>
+        <v>1163</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9157,13 +9160,13 @@
         <v>46311</v>
       </c>
       <c r="B20" s="58" t="s">
-        <v>1163</v>
+        <v>1164</v>
       </c>
       <c r="C20" s="58" t="s">
-        <v>1164</v>
+        <v>1165</v>
       </c>
       <c r="D20" s="58" t="s">
-        <v>1165</v>
+        <v>1166</v>
       </c>
     </row>
   </sheetData>
@@ -10500,7 +10503,7 @@
         <v>277</v>
       </c>
     </row>
-    <row r="136" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="136" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A136" s="42" t="s">
         <v>278</v>
       </c>
@@ -10511,7 +10514,7 @@
         <v>279</v>
       </c>
     </row>
-    <row r="137" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="137" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A137" s="50" t="s">
         <v>280</v>
       </c>
@@ -14527,7 +14530,7 @@
         <v>775</v>
       </c>
       <c r="I63" s="69" t="s">
-        <v>640</v>
+        <v>626</v>
       </c>
       <c r="J63" s="27" t="s">
         <v>797</v>

</xml_diff>

<commit_message>
Storm bail tuning by difficulty, storm practice key, seeded ring tests; plan: G0 and G1 passed, Production statuses; README
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018inbrQHz2eFfbj9ny1keZA
</commit_message>
<xml_diff>
--- a/docs/Vinland_Game_Development_Plan.xlsx
+++ b/docs/Vinland_Game_Development_Plan.xlsx
@@ -86,7 +86,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1920" uniqueCount="1197">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1920" uniqueCount="1198">
   <si>
     <t xml:space="preserve">VINLAND</t>
   </si>
@@ -2056,60 +2056,60 @@
     <t xml:space="preserve">Must</t>
   </si>
   <si>
+    <t xml:space="preserve">Done</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Someone who did not design it finds a fix and argues about the hold.  [Digital ring prototype stood in for the paper test.]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F42</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Engine bake-off: ring prototype in both engines</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tech</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Engineering</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Engine chosen by week 2 on ring feel and haptic API, not feature lists.  [Godot 4.3 chosen 17 Oct 2026 without a bake-off: free, exports PC and web, builds headless for automated tests.]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F43</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Source control, build pipeline, tagged builds</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Every playtest build is reproducible from a tag.  [Repo, tagged-quality builds, headless tests, Windows and Web exports.]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F44</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Art style target: one sea, one camp, one UI frame</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Art</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Not started</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Three paintovers approved: wood, wool, and a ring, not chrome.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hold and ration model</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Economy</t>
+  </si>
+  <si>
     <t xml:space="preserve">In progress</t>
   </si>
   <si>
-    <t xml:space="preserve">Someone who did not design it finds a fix and argues about the hold.  [Digital ring prototype stands in for the paper test; needs a tester who did not design it.]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">F42</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Engine bake-off: ring prototype in both engines</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tech</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Engineering</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Done</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Engine chosen by week 2 on ring feel and haptic API, not feature lists.  [Godot 4.3 chosen 17 Oct 2026 without a bake-off: free, exports PC and web, builds headless for automated tests.]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">F43</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Source control, build pipeline, tagged builds</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Every playtest build is reproducible from a tag.  [Git repo, tagged builds, headless tests and Windows/Web exports work. Push to GitHub waits on repo access.]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">F44</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Art style target: one sea, one camp, one UI frame</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Art</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Not started</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Three paintovers approved: wood, wool, and a ring, not chrome.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hold and ration model</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Economy</t>
-  </si>
-  <si>
     <t xml:space="preserve">Cargo units, rations, and spoilage read from Assumptions knobs; no literals in code.  [Hold, rations, spoilage and animal fodder run from knobs; HoldCheck arithmetic reproduced and tested.]</t>
   </si>
   <si>
@@ -2125,7 +2125,7 @@
     <t xml:space="preserve">Star ring mini-game</t>
   </si>
   <si>
-    <t xml:space="preserve">Fix result (clean, partial, none) feeds drift; playable with haptics off.  [Prototype playable: 5 conditions, haptics with visual twin, run log CSV. Needs human playtests.]</t>
+    <t xml:space="preserve">Fix result (clean, partial, none) feeds drift; playable with haptics off.  [Star ring passed the slice playtest after the difficulty retune.]</t>
   </si>
   <si>
     <t xml:space="preserve">Sun board mini-game</t>
@@ -2137,7 +2137,7 @@
     <t xml:space="preserve">Hand-line fishing</t>
   </si>
   <si>
-    <t xml:space="preserve">A bite reads through the trigger; a cut line keeps the hook.  [Playable: depth by stick, nibbles, two-beat bite, set on the ease, haul under line strain, snap, cut; hooks are a stock. Bots: skilled watch ~19.5 person-days.]</t>
+    <t xml:space="preserve">A bite reads through the trigger; a cut line keeps the hook.  [Hand line passed the slice playtest after the difficulty retune.]</t>
   </si>
   <si>
     <t xml:space="preserve">F06</t>
@@ -2146,13 +2146,13 @@
     <t xml:space="preserve">One camp day loop</t>
   </si>
   <si>
-    <t xml:space="preserve">Morning job queue, one verb, evening tally that changes the hold.  [Playable: morning job board, you play the joint or the hand line, evening tally, a week at a time, G1 checklist at autumn.]</t>
+    <t xml:space="preserve">Morning job queue, one verb, evening tally that changes the hold.  [Camp day loop shipped in the slice and extended to a full year.]</t>
   </si>
   <si>
     <t xml:space="preserve">Joint construction</t>
   </si>
   <si>
-    <t xml:space="preserve">Grain reported on RT; a split log costs the day.  [Playable: brace, set the peg, drive by trigger depth; rain lowers the grain cap. Bots: steady 100%, full force 0%, timid 0%, no brace 22%.]</t>
+    <t xml:space="preserve">Grain reported on RT; a split log costs the day.  [Joint passed the slice playtest after the difficulty retune.]</t>
   </si>
   <si>
     <t xml:space="preserve">F08</t>
@@ -2236,7 +2236,7 @@
     <t xml:space="preserve">Seven cards shuffled per leg; each card offers a verb or takes one away.  [Seven cards plus fair wind, weighted per leg; card shown at each dawn.]</t>
   </si>
   <si>
-    <t xml:space="preserve">No sky game in a storm: hull check, then bail rhythm.</t>
+    <t xml:space="preserve">No sky game in a storm: hull check, then bail rhythm.  [Playable: find the leak, bail on the beat, wave sets with early rumble. Novice keyboard holds 100/92/42% (Forgiving/Standard/Hard).]</t>
   </si>
   <si>
     <t xml:space="preserve">F11</t>
@@ -2266,13 +2266,13 @@
     <t xml:space="preserve">Drying and smoke rack</t>
   </si>
   <si>
-    <t xml:space="preserve">Two fair days turn fresh fish into a food unit.</t>
+    <t xml:space="preserve">Two fair days turn fresh fish into a food unit.  [Smoke-and-dry job turns surplus fresh fish into stores on fair days (90% kept). Rack mini-game (MG9) still to come.]</t>
   </si>
   <si>
     <t xml:space="preserve">Livestock, milk, hay</t>
   </si>
   <si>
-    <t xml:space="preserve">Hay cut in late summer or the byre is a tomb.  [Milk from fed cows; hay job opens 1 August. Byre and winter feeding still to come.]</t>
+    <t xml:space="preserve">Hay cut in late summer or the byre is a tomb.  [Milk from fed cows; hay cut August to mid-October; herd eats hay all winter; no hay kills animals.]</t>
   </si>
   <si>
     <t xml:space="preserve">F17</t>
@@ -2281,7 +2281,7 @@
     <t xml:space="preserve">Byre, longhouse, booths</t>
   </si>
   <si>
-    <t xml:space="preserve">Three buildings raised with the joint and lift verbs; no tech tree.  [Booth plots and the longhouse as a build queue with visible stages (placeholder drawings).]</t>
+    <t xml:space="preserve">Three buildings raised with the joint and lift verbs; no tech tree.  [Build queue: three booths, the longhouse (540 builder-days), the byre (160). Placeholder drawings.]</t>
   </si>
   <si>
     <t xml:space="preserve">Lift and slipway</t>
@@ -2353,7 +2353,7 @@
     <t xml:space="preserve">Winter camp loop and starvation check</t>
   </si>
   <si>
-    <t xml:space="preserve">Each winter week checks hay, food, and shelter; starvation ends the run.</t>
+    <t xml:space="preserve">Each winter week checks hay, food, and shelter; starvation ends the run.  [Seasons and years; first snow 1 Nov, thaw 20 Apr; winter shelter, work, sickness and cold deaths. Year sweeps: a planning camp loses no one, a summer-only camp about 8.]</t>
   </si>
   <si>
     <t xml:space="preserve">F48</t>
@@ -2383,7 +2383,7 @@
     <t xml:space="preserve">Save system</t>
   </si>
   <si>
-    <t xml:space="preserve">Watch-level autosave at sea, day-level in camp, three rolling slots.</t>
+    <t xml:space="preserve">Watch-level autosave at sea, day-level in camp, three rolling slots.  [Autosave every watch at sea and every day ashore, three rolling slots written via temp file, exact-replay loads, Continue on the title.]</t>
   </si>
   <si>
     <t xml:space="preserve">F51</t>
@@ -2950,7 +2950,10 @@
     <t xml:space="preserve">Pillars signed. Paper prototype of the ring judged fun by someone who did not design it.</t>
   </si>
   <si>
-    <t xml:space="preserve">Notes from the table session</t>
+    <t xml:space="preserve">Digital ring prototype, 17 Oct 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Passed</t>
   </si>
   <si>
     <t xml:space="preserve">F41, F42, F43, F44</t>
@@ -2962,7 +2965,7 @@
     <t xml:space="preserve">Slice: leave a fjord, miss a fix, fish, dry nothing, build one joint, see the hold change.</t>
   </si>
   <si>
-    <t xml:space="preserve">Build tag slice-1</t>
+    <t xml:space="preserve">Slice build v2, playtest 17 Oct 2026 ("much better")</t>
   </si>
   <si>
     <t xml:space="preserve">F01, F02, F03, F04, F05, F06, F07, F08, F35, F36, F37, F38, F39, F40, F61</t>
@@ -4881,11 +4884,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="22413173"/>
-        <c:axId val="37001983"/>
+        <c:axId val="58729634"/>
+        <c:axId val="67663476"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="22413173"/>
+        <c:axId val="58729634"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4917,7 +4920,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="37001983"/>
+        <c:crossAx val="67663476"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -4925,7 +4928,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="37001983"/>
+        <c:axId val="67663476"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5001,7 +5004,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="22413173"/>
+        <c:crossAx val="58729634"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -5040,9 +5043,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>743400</xdr:colOff>
+      <xdr:colOff>743040</xdr:colOff>
       <xdr:row>40</xdr:row>
-      <xdr:rowOff>59760</xdr:rowOff>
+      <xdr:rowOff>59400</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -5051,7 +5054,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="0" y="6562800"/>
-        <a:ext cx="5395320" cy="2155320"/>
+        <a:ext cx="5394960" cy="2154960"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -5966,7 +5969,7 @@
       </c>
       <c r="B55" s="5" t="str">
         <f aca="false">COUNTIF(Backlog!I5:I80,"Done")&amp;" of "&amp;COUNTA(Backlog!A5:A80)</f>
-        <v>1 of 65</v>
+        <v>7 of 65</v>
       </c>
       <c r="C55" s="31" t="s">
         <v>68</v>
@@ -5988,7 +5991,7 @@
       </c>
       <c r="B56" s="38" t="n">
         <f aca="false">Backlog!G86</f>
-        <v>0.0261437908496732</v>
+        <v>0.169934640522876</v>
       </c>
       <c r="C56" s="34" t="s">
         <v>71</v>
@@ -6010,7 +6013,7 @@
       </c>
       <c r="B57" s="5" t="str">
         <f aca="false">COUNTIF(Milestones!F5:F10,"Passed")&amp;" of 6"</f>
-        <v>0 of 6</v>
+        <v>2 of 6</v>
       </c>
       <c r="C57" s="31" t="s">
         <v>73</v>
@@ -6247,7 +6250,7 @@
     </row>
     <row r="7" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="26" t="s">
-        <v>669</v>
+        <v>668</v>
       </c>
       <c r="B7" s="89" t="n">
         <f aca="false">Assumptions!B28</f>
@@ -6487,7 +6490,7 @@
         <v>661</v>
       </c>
       <c r="E14" s="9" t="s">
-        <v>669</v>
+        <v>668</v>
       </c>
       <c r="F14" s="9" t="s">
         <v>761</v>
@@ -7505,13 +7508,13 @@
         <v>322</v>
       </c>
       <c r="F5" s="69" t="s">
-        <v>670</v>
+        <v>955</v>
       </c>
       <c r="G5" s="27" t="s">
-        <v>955</v>
+        <v>956</v>
       </c>
       <c r="H5" s="27" t="s">
-        <v>956</v>
+        <v>957</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7523,22 +7526,22 @@
         <v>46453</v>
       </c>
       <c r="C6" s="58" t="s">
-        <v>957</v>
+        <v>958</v>
       </c>
       <c r="D6" s="58" t="s">
-        <v>958</v>
+        <v>959</v>
       </c>
       <c r="E6" s="58" t="s">
         <v>661</v>
       </c>
       <c r="F6" s="69" t="s">
-        <v>670</v>
+        <v>955</v>
       </c>
       <c r="G6" s="58" t="s">
-        <v>959</v>
+        <v>960</v>
       </c>
       <c r="H6" s="58" t="s">
-        <v>960</v>
+        <v>961</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7550,22 +7553,22 @@
         <v>46579</v>
       </c>
       <c r="C7" s="27" t="s">
-        <v>961</v>
+        <v>962</v>
       </c>
       <c r="D7" s="27" t="s">
-        <v>962</v>
+        <v>963</v>
       </c>
       <c r="E7" s="27" t="s">
         <v>322</v>
       </c>
       <c r="F7" s="69" t="s">
-        <v>670</v>
+        <v>673</v>
       </c>
       <c r="G7" s="27" t="s">
-        <v>963</v>
+        <v>964</v>
       </c>
       <c r="H7" s="27" t="s">
-        <v>964</v>
+        <v>965</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7577,22 +7580,22 @@
         <v>46621</v>
       </c>
       <c r="C8" s="58" t="s">
-        <v>965</v>
+        <v>966</v>
       </c>
       <c r="D8" s="58" t="s">
-        <v>966</v>
+        <v>967</v>
       </c>
       <c r="E8" s="58" t="s">
         <v>100</v>
       </c>
       <c r="F8" s="69" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="G8" s="58" t="s">
-        <v>967</v>
+        <v>968</v>
       </c>
       <c r="H8" s="58" t="s">
-        <v>968</v>
+        <v>969</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7604,22 +7607,22 @@
         <v>46663</v>
       </c>
       <c r="C9" s="27" t="s">
-        <v>969</v>
+        <v>970</v>
       </c>
       <c r="D9" s="27" t="s">
-        <v>970</v>
+        <v>971</v>
       </c>
       <c r="E9" s="27" t="s">
         <v>816</v>
       </c>
       <c r="F9" s="69" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="G9" s="27" t="s">
-        <v>971</v>
+        <v>972</v>
       </c>
       <c r="H9" s="27" t="s">
-        <v>972</v>
+        <v>973</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7631,19 +7634,19 @@
         <v>46691</v>
       </c>
       <c r="C10" s="58" t="s">
-        <v>973</v>
+        <v>974</v>
       </c>
       <c r="D10" s="58" t="s">
-        <v>974</v>
+        <v>975</v>
       </c>
       <c r="E10" s="58" t="s">
         <v>100</v>
       </c>
       <c r="F10" s="69" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="G10" s="58" t="s">
-        <v>975</v>
+        <v>976</v>
       </c>
       <c r="H10" s="58" t="s">
         <v>427</v>
@@ -7651,7 +7654,7 @@
     </row>
     <row r="12" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="54" t="s">
-        <v>976</v>
+        <v>977</v>
       </c>
       <c r="B12" s="54"/>
       <c r="C12" s="54"/>
@@ -7731,7 +7734,7 @@
     </row>
     <row r="2" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>977</v>
+        <v>978</v>
       </c>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
@@ -7748,28 +7751,28 @@
         <v>313</v>
       </c>
       <c r="B4" s="57" t="s">
-        <v>978</v>
+        <v>979</v>
       </c>
       <c r="C4" s="57" t="s">
-        <v>979</v>
+        <v>980</v>
       </c>
       <c r="D4" s="57" t="s">
-        <v>980</v>
+        <v>981</v>
       </c>
       <c r="E4" s="57" t="s">
         <v>463</v>
       </c>
       <c r="F4" s="57" t="s">
-        <v>981</v>
+        <v>982</v>
       </c>
       <c r="G4" s="57" t="s">
         <v>649</v>
       </c>
       <c r="H4" s="57" t="s">
-        <v>982</v>
+        <v>983</v>
       </c>
       <c r="I4" s="9" t="s">
-        <v>983</v>
+        <v>984</v>
       </c>
       <c r="J4" s="9" t="s">
         <v>44</v>
@@ -7777,10 +7780,10 @@
     </row>
     <row r="5" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="58" t="s">
-        <v>984</v>
+        <v>985</v>
       </c>
       <c r="B5" s="58" t="s">
-        <v>985</v>
+        <v>986</v>
       </c>
       <c r="C5" s="43" t="n">
         <v>3</v>
@@ -7793,7 +7796,7 @@
         <v>15</v>
       </c>
       <c r="F5" s="58" t="s">
-        <v>986</v>
+        <v>987</v>
       </c>
       <c r="G5" s="58" t="s">
         <v>322</v>
@@ -7802,18 +7805,18 @@
         <v>873</v>
       </c>
       <c r="I5" s="58" t="s">
-        <v>987</v>
+        <v>988</v>
       </c>
       <c r="J5" s="69" t="s">
-        <v>988</v>
+        <v>989</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="58" t="s">
-        <v>989</v>
+        <v>990</v>
       </c>
       <c r="B6" s="58" t="s">
-        <v>990</v>
+        <v>991</v>
       </c>
       <c r="C6" s="43" t="n">
         <v>3</v>
@@ -7826,7 +7829,7 @@
         <v>12</v>
       </c>
       <c r="F6" s="58" t="s">
-        <v>991</v>
+        <v>992</v>
       </c>
       <c r="G6" s="58" t="s">
         <v>322</v>
@@ -7835,18 +7838,18 @@
         <v>873</v>
       </c>
       <c r="I6" s="58" t="s">
-        <v>992</v>
+        <v>993</v>
       </c>
       <c r="J6" s="69" t="s">
-        <v>993</v>
+        <v>994</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="58" t="s">
-        <v>994</v>
+        <v>995</v>
       </c>
       <c r="B7" s="58" t="s">
-        <v>995</v>
+        <v>996</v>
       </c>
       <c r="C7" s="43" t="n">
         <v>2</v>
@@ -7859,7 +7862,7 @@
         <v>8</v>
       </c>
       <c r="F7" s="58" t="s">
-        <v>996</v>
+        <v>997</v>
       </c>
       <c r="G7" s="58" t="s">
         <v>661</v>
@@ -7868,18 +7871,18 @@
         <v>885</v>
       </c>
       <c r="I7" s="58" t="s">
-        <v>997</v>
+        <v>998</v>
       </c>
       <c r="J7" s="69" t="s">
-        <v>993</v>
+        <v>994</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="58" t="s">
-        <v>998</v>
+        <v>999</v>
       </c>
       <c r="B8" s="58" t="s">
-        <v>999</v>
+        <v>1000</v>
       </c>
       <c r="C8" s="43" t="n">
         <v>4</v>
@@ -7892,7 +7895,7 @@
         <v>12</v>
       </c>
       <c r="F8" s="58" t="s">
-        <v>1000</v>
+        <v>1001</v>
       </c>
       <c r="G8" s="58" t="s">
         <v>100</v>
@@ -7901,18 +7904,18 @@
         <v>877</v>
       </c>
       <c r="I8" s="58" t="s">
-        <v>1001</v>
+        <v>1002</v>
       </c>
       <c r="J8" s="69" t="s">
-        <v>993</v>
+        <v>994</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="58" t="s">
-        <v>1002</v>
+        <v>1003</v>
       </c>
       <c r="B9" s="58" t="s">
-        <v>1003</v>
+        <v>1004</v>
       </c>
       <c r="C9" s="43" t="n">
         <v>2</v>
@@ -7925,27 +7928,27 @@
         <v>6</v>
       </c>
       <c r="F9" s="58" t="s">
-        <v>1004</v>
+        <v>1005</v>
       </c>
       <c r="G9" s="58" t="s">
-        <v>669</v>
+        <v>668</v>
       </c>
       <c r="H9" s="58" t="s">
         <v>877</v>
       </c>
       <c r="I9" s="58" t="s">
-        <v>1005</v>
+        <v>1006</v>
       </c>
       <c r="J9" s="69" t="s">
-        <v>993</v>
+        <v>994</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="58" t="s">
-        <v>1006</v>
+        <v>1007</v>
       </c>
       <c r="B10" s="58" t="s">
-        <v>1007</v>
+        <v>1008</v>
       </c>
       <c r="C10" s="43" t="n">
         <v>2</v>
@@ -7958,7 +7961,7 @@
         <v>10</v>
       </c>
       <c r="F10" s="58" t="s">
-        <v>1008</v>
+        <v>1009</v>
       </c>
       <c r="G10" s="58" t="s">
         <v>322</v>
@@ -7967,18 +7970,18 @@
         <v>877</v>
       </c>
       <c r="I10" s="58" t="s">
-        <v>1009</v>
+        <v>1010</v>
       </c>
       <c r="J10" s="69" t="s">
-        <v>993</v>
+        <v>994</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="58" t="s">
-        <v>1010</v>
+        <v>1011</v>
       </c>
       <c r="B11" s="58" t="s">
-        <v>1011</v>
+        <v>1012</v>
       </c>
       <c r="C11" s="43" t="n">
         <v>3</v>
@@ -7991,7 +7994,7 @@
         <v>12</v>
       </c>
       <c r="F11" s="58" t="s">
-        <v>1012</v>
+        <v>1013</v>
       </c>
       <c r="G11" s="58" t="s">
         <v>100</v>
@@ -8000,18 +8003,18 @@
         <v>881</v>
       </c>
       <c r="I11" s="58" t="s">
-        <v>1013</v>
+        <v>1014</v>
       </c>
       <c r="J11" s="69" t="s">
-        <v>993</v>
+        <v>994</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="58" t="s">
-        <v>1014</v>
+        <v>1015</v>
       </c>
       <c r="B12" s="58" t="s">
-        <v>1015</v>
+        <v>1016</v>
       </c>
       <c r="C12" s="43" t="n">
         <v>2</v>
@@ -8024,7 +8027,7 @@
         <v>8</v>
       </c>
       <c r="F12" s="58" t="s">
-        <v>1016</v>
+        <v>1017</v>
       </c>
       <c r="G12" s="58" t="s">
         <v>661</v>
@@ -8033,18 +8036,18 @@
         <v>869</v>
       </c>
       <c r="I12" s="58" t="s">
-        <v>1017</v>
+        <v>1018</v>
       </c>
       <c r="J12" s="69" t="s">
-        <v>993</v>
+        <v>994</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="58" t="s">
-        <v>1018</v>
+        <v>1019</v>
       </c>
       <c r="B13" s="58" t="s">
-        <v>1019</v>
+        <v>1020</v>
       </c>
       <c r="C13" s="43" t="n">
         <v>2</v>
@@ -8057,7 +8060,7 @@
         <v>4</v>
       </c>
       <c r="F13" s="58" t="s">
-        <v>1020</v>
+        <v>1021</v>
       </c>
       <c r="G13" s="58" t="s">
         <v>322</v>
@@ -8066,18 +8069,18 @@
         <v>869</v>
       </c>
       <c r="I13" s="58" t="s">
-        <v>1021</v>
+        <v>1022</v>
       </c>
       <c r="J13" s="69" t="s">
-        <v>993</v>
+        <v>994</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="58" t="s">
-        <v>1022</v>
+        <v>1023</v>
       </c>
       <c r="B14" s="58" t="s">
-        <v>1023</v>
+        <v>1024</v>
       </c>
       <c r="C14" s="43" t="n">
         <v>3</v>
@@ -8090,7 +8093,7 @@
         <v>12</v>
       </c>
       <c r="F14" s="58" t="s">
-        <v>1024</v>
+        <v>1025</v>
       </c>
       <c r="G14" s="58" t="s">
         <v>322</v>
@@ -8099,18 +8102,18 @@
         <v>881</v>
       </c>
       <c r="I14" s="58" t="s">
-        <v>1025</v>
+        <v>1026</v>
       </c>
       <c r="J14" s="69" t="s">
-        <v>993</v>
+        <v>994</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="58" t="s">
-        <v>1026</v>
+        <v>1027</v>
       </c>
       <c r="B15" s="58" t="s">
-        <v>1027</v>
+        <v>1028</v>
       </c>
       <c r="C15" s="43" t="n">
         <v>3</v>
@@ -8123,7 +8126,7 @@
         <v>15</v>
       </c>
       <c r="F15" s="58" t="s">
-        <v>1028</v>
+        <v>1029</v>
       </c>
       <c r="G15" s="58" t="s">
         <v>322</v>
@@ -8132,18 +8135,18 @@
         <v>877</v>
       </c>
       <c r="I15" s="58" t="s">
-        <v>1029</v>
+        <v>1030</v>
       </c>
       <c r="J15" s="69" t="s">
-        <v>993</v>
+        <v>994</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="58" t="s">
-        <v>1030</v>
+        <v>1031</v>
       </c>
       <c r="B16" s="58" t="s">
-        <v>1031</v>
+        <v>1032</v>
       </c>
       <c r="C16" s="43" t="n">
         <v>4</v>
@@ -8156,7 +8159,7 @@
         <v>16</v>
       </c>
       <c r="F16" s="58" t="s">
-        <v>1032</v>
+        <v>1033</v>
       </c>
       <c r="G16" s="58" t="s">
         <v>100</v>
@@ -8165,18 +8168,18 @@
         <v>873</v>
       </c>
       <c r="I16" s="58" t="s">
-        <v>1033</v>
+        <v>1034</v>
       </c>
       <c r="J16" s="69" t="s">
-        <v>993</v>
+        <v>994</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="58" t="s">
-        <v>1034</v>
+        <v>1035</v>
       </c>
       <c r="B17" s="58" t="s">
-        <v>1035</v>
+        <v>1036</v>
       </c>
       <c r="C17" s="43" t="n">
         <v>3</v>
@@ -8189,7 +8192,7 @@
         <v>12</v>
       </c>
       <c r="F17" s="58" t="s">
-        <v>1036</v>
+        <v>1037</v>
       </c>
       <c r="G17" s="58" t="s">
         <v>100</v>
@@ -8198,18 +8201,18 @@
         <v>877</v>
       </c>
       <c r="I17" s="58" t="s">
-        <v>1037</v>
+        <v>1038</v>
       </c>
       <c r="J17" s="69" t="s">
-        <v>993</v>
+        <v>994</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="58" t="s">
-        <v>1038</v>
+        <v>1039</v>
       </c>
       <c r="B18" s="58" t="s">
-        <v>1039</v>
+        <v>1040</v>
       </c>
       <c r="C18" s="43" t="n">
         <v>2</v>
@@ -8222,7 +8225,7 @@
         <v>6</v>
       </c>
       <c r="F18" s="58" t="s">
-        <v>1040</v>
+        <v>1041</v>
       </c>
       <c r="G18" s="58" t="s">
         <v>322</v>
@@ -8231,18 +8234,18 @@
         <v>885</v>
       </c>
       <c r="I18" s="58" t="s">
-        <v>1041</v>
+        <v>1042</v>
       </c>
       <c r="J18" s="69" t="s">
-        <v>993</v>
+        <v>994</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="58" t="s">
-        <v>1042</v>
+        <v>1043</v>
       </c>
       <c r="B19" s="58" t="s">
-        <v>1043</v>
+        <v>1044</v>
       </c>
       <c r="C19" s="43" t="n">
         <v>2</v>
@@ -8255,7 +8258,7 @@
         <v>8</v>
       </c>
       <c r="F19" s="58" t="s">
-        <v>1044</v>
+        <v>1045</v>
       </c>
       <c r="G19" s="58" t="s">
         <v>661</v>
@@ -8264,18 +8267,18 @@
         <v>877</v>
       </c>
       <c r="I19" s="58" t="s">
-        <v>1045</v>
+        <v>1046</v>
       </c>
       <c r="J19" s="69" t="s">
-        <v>993</v>
+        <v>994</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="58" t="s">
-        <v>1046</v>
+        <v>1047</v>
       </c>
       <c r="B20" s="58" t="s">
-        <v>1047</v>
+        <v>1048</v>
       </c>
       <c r="C20" s="43" t="n">
         <v>3</v>
@@ -8288,7 +8291,7 @@
         <v>15</v>
       </c>
       <c r="F20" s="58" t="s">
-        <v>1048</v>
+        <v>1049</v>
       </c>
       <c r="G20" s="58" t="s">
         <v>100</v>
@@ -8297,10 +8300,10 @@
         <v>873</v>
       </c>
       <c r="I20" s="58" t="s">
-        <v>1049</v>
+        <v>1050</v>
       </c>
       <c r="J20" s="69" t="s">
-        <v>993</v>
+        <v>994</v>
       </c>
     </row>
   </sheetData>
@@ -8378,7 +8381,7 @@
     </row>
     <row r="2" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>1050</v>
+        <v>1051</v>
       </c>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
@@ -8389,16 +8392,16 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="57" t="s">
-        <v>1051</v>
+        <v>1052</v>
       </c>
       <c r="B4" s="57" t="s">
-        <v>1052</v>
+        <v>1053</v>
       </c>
       <c r="C4" s="57" t="s">
-        <v>1053</v>
+        <v>1054</v>
       </c>
       <c r="D4" s="57" t="s">
-        <v>1054</v>
+        <v>1055</v>
       </c>
       <c r="E4" s="57" t="s">
         <v>95</v>
@@ -8407,30 +8410,30 @@
         <v>649</v>
       </c>
       <c r="G4" s="9" t="s">
-        <v>1055</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="27" t="s">
-        <v>1056</v>
+        <v>1057</v>
       </c>
       <c r="B5" s="27" t="s">
-        <v>1057</v>
+        <v>1058</v>
       </c>
       <c r="C5" s="27" t="s">
-        <v>1058</v>
+        <v>1059</v>
       </c>
       <c r="D5" s="27" t="s">
-        <v>1059</v>
+        <v>1060</v>
       </c>
       <c r="E5" s="27" t="s">
-        <v>1060</v>
+        <v>1061</v>
       </c>
       <c r="F5" s="27" t="s">
-        <v>669</v>
+        <v>668</v>
       </c>
       <c r="G5" s="27" t="s">
-        <v>1061</v>
+        <v>1062</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8438,68 +8441,68 @@
         <v>621</v>
       </c>
       <c r="B6" s="58" t="s">
-        <v>1062</v>
+        <v>1063</v>
       </c>
       <c r="C6" s="58" t="s">
-        <v>1063</v>
+        <v>1064</v>
       </c>
       <c r="D6" s="58" t="s">
-        <v>1064</v>
+        <v>1065</v>
       </c>
       <c r="E6" s="58" t="s">
-        <v>1065</v>
+        <v>1066</v>
       </c>
       <c r="F6" s="58" t="s">
-        <v>1066</v>
+        <v>1067</v>
       </c>
       <c r="G6" s="58" t="s">
-        <v>1067</v>
+        <v>1068</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="27" t="s">
+        <v>1069</v>
+      </c>
+      <c r="B7" s="27" t="s">
+        <v>1070</v>
+      </c>
+      <c r="C7" s="27" t="s">
+        <v>1071</v>
+      </c>
+      <c r="D7" s="27" t="s">
+        <v>1072</v>
+      </c>
+      <c r="E7" s="27" t="s">
+        <v>1073</v>
+      </c>
+      <c r="F7" s="27" t="s">
+        <v>668</v>
+      </c>
+      <c r="G7" s="27" t="s">
         <v>1068</v>
-      </c>
-      <c r="B7" s="27" t="s">
-        <v>1069</v>
-      </c>
-      <c r="C7" s="27" t="s">
-        <v>1070</v>
-      </c>
-      <c r="D7" s="27" t="s">
-        <v>1071</v>
-      </c>
-      <c r="E7" s="27" t="s">
-        <v>1072</v>
-      </c>
-      <c r="F7" s="27" t="s">
-        <v>669</v>
-      </c>
-      <c r="G7" s="27" t="s">
-        <v>1067</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="58" t="s">
-        <v>1073</v>
+        <v>1074</v>
       </c>
       <c r="B8" s="58" t="s">
-        <v>1074</v>
+        <v>1075</v>
       </c>
       <c r="C8" s="58" t="s">
-        <v>1075</v>
+        <v>1076</v>
       </c>
       <c r="D8" s="58" t="s">
-        <v>1076</v>
+        <v>1077</v>
       </c>
       <c r="E8" s="58" t="s">
-        <v>1077</v>
+        <v>1078</v>
       </c>
       <c r="F8" s="58" t="s">
-        <v>669</v>
+        <v>668</v>
       </c>
       <c r="G8" s="58" t="s">
-        <v>1078</v>
+        <v>1079</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8507,22 +8510,22 @@
         <v>506</v>
       </c>
       <c r="B9" s="27" t="s">
-        <v>1079</v>
+        <v>1080</v>
       </c>
       <c r="C9" s="27" t="s">
-        <v>1080</v>
+        <v>1081</v>
       </c>
       <c r="D9" s="27" t="s">
-        <v>1081</v>
+        <v>1082</v>
       </c>
       <c r="E9" s="27" t="s">
-        <v>1082</v>
+        <v>1083</v>
       </c>
       <c r="F9" s="27" t="s">
-        <v>669</v>
+        <v>668</v>
       </c>
       <c r="G9" s="27" t="s">
-        <v>1083</v>
+        <v>1084</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8530,22 +8533,22 @@
         <v>697</v>
       </c>
       <c r="B10" s="58" t="s">
-        <v>1084</v>
+        <v>1085</v>
       </c>
       <c r="C10" s="58" t="s">
-        <v>1085</v>
+        <v>1086</v>
       </c>
       <c r="D10" s="58" t="s">
         <v>819</v>
       </c>
       <c r="E10" s="58" t="s">
-        <v>1086</v>
+        <v>1087</v>
       </c>
       <c r="F10" s="58" t="s">
-        <v>669</v>
+        <v>668</v>
       </c>
       <c r="G10" s="58" t="s">
-        <v>1087</v>
+        <v>1088</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8553,22 +8556,22 @@
         <v>761</v>
       </c>
       <c r="B11" s="27" t="s">
-        <v>1088</v>
+        <v>1089</v>
       </c>
       <c r="C11" s="27" t="s">
-        <v>1089</v>
+        <v>1090</v>
       </c>
       <c r="D11" s="27" t="s">
-        <v>1090</v>
+        <v>1091</v>
       </c>
       <c r="E11" s="27" t="s">
-        <v>1091</v>
+        <v>1092</v>
       </c>
       <c r="F11" s="27" t="s">
         <v>761</v>
       </c>
       <c r="G11" s="27" t="s">
-        <v>1092</v>
+        <v>1093</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8576,91 +8579,91 @@
         <v>780</v>
       </c>
       <c r="B12" s="58" t="s">
-        <v>1093</v>
+        <v>1094</v>
       </c>
       <c r="C12" s="58" t="s">
-        <v>1094</v>
+        <v>1095</v>
       </c>
       <c r="D12" s="58" t="s">
-        <v>1095</v>
+        <v>1096</v>
       </c>
       <c r="E12" s="58" t="s">
-        <v>1096</v>
+        <v>1097</v>
       </c>
       <c r="F12" s="58" t="s">
         <v>322</v>
       </c>
       <c r="G12" s="58" t="s">
-        <v>1067</v>
+        <v>1068</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="27" t="s">
-        <v>1097</v>
+        <v>1098</v>
       </c>
       <c r="B13" s="27" t="s">
-        <v>1098</v>
+        <v>1099</v>
       </c>
       <c r="C13" s="27" t="s">
-        <v>1099</v>
+        <v>1100</v>
       </c>
       <c r="D13" s="27" t="s">
-        <v>1100</v>
+        <v>1101</v>
       </c>
       <c r="E13" s="27" t="s">
-        <v>1101</v>
+        <v>1102</v>
       </c>
       <c r="F13" s="27" t="s">
         <v>661</v>
       </c>
       <c r="G13" s="27" t="s">
-        <v>1067</v>
+        <v>1068</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="58" t="s">
-        <v>1102</v>
+        <v>1103</v>
       </c>
       <c r="B14" s="58" t="s">
-        <v>1103</v>
+        <v>1104</v>
       </c>
       <c r="C14" s="58" t="s">
-        <v>1104</v>
+        <v>1105</v>
       </c>
       <c r="D14" s="58" t="s">
-        <v>1105</v>
+        <v>1106</v>
       </c>
       <c r="E14" s="58" t="s">
-        <v>1106</v>
+        <v>1107</v>
       </c>
       <c r="F14" s="58" t="s">
         <v>100</v>
       </c>
       <c r="G14" s="58" t="s">
-        <v>1107</v>
+        <v>1108</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="27" t="s">
-        <v>1108</v>
+        <v>1109</v>
       </c>
       <c r="B15" s="27" t="s">
-        <v>1109</v>
+        <v>1110</v>
       </c>
       <c r="C15" s="27" t="s">
-        <v>1110</v>
+        <v>1111</v>
       </c>
       <c r="D15" s="27" t="s">
-        <v>1111</v>
+        <v>1112</v>
       </c>
       <c r="E15" s="27" t="s">
-        <v>1112</v>
+        <v>1113</v>
       </c>
       <c r="F15" s="27" t="s">
         <v>100</v>
       </c>
       <c r="G15" s="27" t="s">
-        <v>1113</v>
+        <v>1114</v>
       </c>
     </row>
   </sheetData>
@@ -8702,7 +8705,7 @@
     </row>
     <row r="2" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>1114</v>
+        <v>1115</v>
       </c>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
@@ -8713,10 +8716,10 @@
         <v>110</v>
       </c>
       <c r="B4" s="57" t="s">
-        <v>1115</v>
+        <v>1116</v>
       </c>
       <c r="C4" s="57" t="s">
-        <v>1116</v>
+        <v>1117</v>
       </c>
       <c r="D4" s="57" t="s">
         <v>649</v>
@@ -8724,10 +8727,10 @@
     </row>
     <row r="5" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="27" t="s">
-        <v>1117</v>
+        <v>1118</v>
       </c>
       <c r="B5" s="27" t="s">
-        <v>1118</v>
+        <v>1119</v>
       </c>
       <c r="C5" s="27" t="s">
         <v>869</v>
@@ -8738,13 +8741,13 @@
     </row>
     <row r="6" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="58" t="s">
-        <v>1119</v>
+        <v>1120</v>
       </c>
       <c r="B6" s="58" t="s">
-        <v>1120</v>
+        <v>1121</v>
       </c>
       <c r="C6" s="58" t="s">
-        <v>1121</v>
+        <v>1122</v>
       </c>
       <c r="D6" s="58" t="s">
         <v>661</v>
@@ -8752,10 +8755,10 @@
     </row>
     <row r="7" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="27" t="s">
-        <v>1122</v>
+        <v>1123</v>
       </c>
       <c r="B7" s="27" t="s">
-        <v>1123</v>
+        <v>1124</v>
       </c>
       <c r="C7" s="27" t="s">
         <v>877</v>
@@ -8766,10 +8769,10 @@
     </row>
     <row r="8" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="58" t="s">
-        <v>1124</v>
+        <v>1125</v>
       </c>
       <c r="B8" s="58" t="s">
-        <v>1125</v>
+        <v>1126</v>
       </c>
       <c r="C8" s="58" t="s">
         <v>873</v>
@@ -8780,10 +8783,10 @@
     </row>
     <row r="9" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="27" t="s">
-        <v>1126</v>
+        <v>1127</v>
       </c>
       <c r="B9" s="27" t="s">
-        <v>1127</v>
+        <v>1128</v>
       </c>
       <c r="C9" s="27" t="s">
         <v>869</v>
@@ -8794,10 +8797,10 @@
     </row>
     <row r="10" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="58" t="s">
-        <v>1128</v>
+        <v>1129</v>
       </c>
       <c r="B10" s="58" t="s">
-        <v>1129</v>
+        <v>1130</v>
       </c>
       <c r="C10" s="58" t="s">
         <v>877</v>
@@ -8808,10 +8811,10 @@
     </row>
     <row r="11" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="27" t="s">
-        <v>1130</v>
+        <v>1131</v>
       </c>
       <c r="B11" s="27" t="s">
-        <v>1131</v>
+        <v>1132</v>
       </c>
       <c r="C11" s="27" t="s">
         <v>885</v>
@@ -8822,10 +8825,10 @@
     </row>
     <row r="12" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="58" t="s">
-        <v>1132</v>
+        <v>1133</v>
       </c>
       <c r="B12" s="58" t="s">
-        <v>1133</v>
+        <v>1134</v>
       </c>
       <c r="C12" s="58" t="s">
         <v>888</v>
@@ -8836,10 +8839,10 @@
     </row>
     <row r="13" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="27" t="s">
-        <v>1134</v>
+        <v>1135</v>
       </c>
       <c r="B13" s="27" t="s">
-        <v>1135</v>
+        <v>1136</v>
       </c>
       <c r="C13" s="27" t="s">
         <v>888</v>
@@ -8850,13 +8853,13 @@
     </row>
     <row r="14" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="58" t="s">
-        <v>1136</v>
+        <v>1137</v>
       </c>
       <c r="B14" s="58" t="s">
-        <v>1137</v>
+        <v>1138</v>
       </c>
       <c r="C14" s="58" t="s">
-        <v>1138</v>
+        <v>1139</v>
       </c>
       <c r="D14" s="58" t="s">
         <v>322</v>
@@ -8864,10 +8867,10 @@
     </row>
     <row r="15" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="27" t="s">
-        <v>1139</v>
+        <v>1140</v>
       </c>
       <c r="B15" s="27" t="s">
-        <v>1140</v>
+        <v>1141</v>
       </c>
       <c r="C15" s="27" t="s">
         <v>873</v>
@@ -8878,7 +8881,7 @@
     </row>
     <row r="16" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="58" t="s">
-        <v>1141</v>
+        <v>1142</v>
       </c>
       <c r="B16" s="58" t="str">
         <f aca="false">"Premium at $"&amp;TEXT(Assumptions!B69,"0.00")&amp;". Launch discount no deeper than the realized-price factor on Assumptions."</f>
@@ -8893,10 +8896,10 @@
     </row>
     <row r="17" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="27" t="s">
-        <v>1142</v>
+        <v>1143</v>
       </c>
       <c r="B17" s="27" t="s">
-        <v>1143</v>
+        <v>1144</v>
       </c>
       <c r="C17" s="27" t="s">
         <v>873</v>
@@ -8910,7 +8913,7 @@
         <v>863</v>
       </c>
       <c r="B18" s="58" t="s">
-        <v>1144</v>
+        <v>1145</v>
       </c>
       <c r="C18" s="58" t="s">
         <v>881</v>
@@ -8921,10 +8924,10 @@
     </row>
     <row r="19" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="27" t="s">
-        <v>1145</v>
+        <v>1146</v>
       </c>
       <c r="B19" s="27" t="s">
-        <v>1146</v>
+        <v>1147</v>
       </c>
       <c r="C19" s="27" t="s">
         <v>885</v>
@@ -8935,10 +8938,10 @@
     </row>
     <row r="20" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="58" t="s">
-        <v>1147</v>
+        <v>1148</v>
       </c>
       <c r="B20" s="58" t="s">
-        <v>1148</v>
+        <v>1149</v>
       </c>
       <c r="C20" s="58" t="s">
         <v>885</v>
@@ -8949,10 +8952,10 @@
     </row>
     <row r="21" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="27" t="s">
-        <v>1149</v>
+        <v>1150</v>
       </c>
       <c r="B21" s="27" t="s">
-        <v>1150</v>
+        <v>1151</v>
       </c>
       <c r="C21" s="27" t="s">
         <v>885</v>
@@ -8963,10 +8966,10 @@
     </row>
     <row r="22" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="58" t="s">
-        <v>1151</v>
+        <v>1152</v>
       </c>
       <c r="B22" s="58" t="s">
-        <v>1152</v>
+        <v>1153</v>
       </c>
       <c r="C22" s="58" t="s">
         <v>888</v>
@@ -9015,7 +9018,7 @@
     </row>
     <row r="2" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>1153</v>
+        <v>1154</v>
       </c>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
@@ -9023,16 +9026,16 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>1154</v>
+        <v>1155</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>1155</v>
+        <v>1156</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>1156</v>
+        <v>1157</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>1157</v>
+        <v>1158</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9040,13 +9043,13 @@
         <v>46311</v>
       </c>
       <c r="B5" s="27" t="s">
-        <v>1158</v>
+        <v>1159</v>
       </c>
       <c r="C5" s="27" t="s">
-        <v>1159</v>
+        <v>1160</v>
       </c>
       <c r="D5" s="27" t="s">
-        <v>1160</v>
+        <v>1161</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9054,13 +9057,13 @@
         <v>46311</v>
       </c>
       <c r="B6" s="58" t="s">
-        <v>1158</v>
+        <v>1159</v>
       </c>
       <c r="C6" s="58" t="s">
-        <v>1161</v>
+        <v>1162</v>
       </c>
       <c r="D6" s="58" t="s">
-        <v>1162</v>
+        <v>1163</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9068,13 +9071,13 @@
         <v>46311</v>
       </c>
       <c r="B7" s="27" t="s">
-        <v>1158</v>
+        <v>1159</v>
       </c>
       <c r="C7" s="27" t="s">
-        <v>1163</v>
+        <v>1164</v>
       </c>
       <c r="D7" s="27" t="s">
-        <v>1164</v>
+        <v>1165</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9085,10 +9088,10 @@
         <v>923</v>
       </c>
       <c r="C8" s="58" t="s">
-        <v>1165</v>
+        <v>1166</v>
       </c>
       <c r="D8" s="58" t="s">
-        <v>1166</v>
+        <v>1167</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9096,13 +9099,13 @@
         <v>46311</v>
       </c>
       <c r="B9" s="27" t="s">
-        <v>1167</v>
+        <v>1168</v>
       </c>
       <c r="C9" s="27" t="s">
-        <v>1168</v>
+        <v>1169</v>
       </c>
       <c r="D9" s="27" t="s">
-        <v>1169</v>
+        <v>1170</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9113,10 +9116,10 @@
         <v>53</v>
       </c>
       <c r="C10" s="58" t="s">
-        <v>1170</v>
+        <v>1171</v>
       </c>
       <c r="D10" s="58" t="s">
-        <v>1171</v>
+        <v>1172</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9124,13 +9127,13 @@
         <v>46311</v>
       </c>
       <c r="B11" s="27" t="s">
-        <v>1172</v>
+        <v>1173</v>
       </c>
       <c r="C11" s="27" t="s">
-        <v>1173</v>
+        <v>1174</v>
       </c>
       <c r="D11" s="27" t="s">
-        <v>1174</v>
+        <v>1175</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9141,10 +9144,10 @@
         <v>402</v>
       </c>
       <c r="C12" s="58" t="s">
-        <v>1175</v>
+        <v>1176</v>
       </c>
       <c r="D12" s="58" t="s">
-        <v>1176</v>
+        <v>1177</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9152,13 +9155,13 @@
         <v>46311</v>
       </c>
       <c r="B13" s="27" t="s">
-        <v>1177</v>
+        <v>1178</v>
       </c>
       <c r="C13" s="27" t="s">
-        <v>1178</v>
+        <v>1179</v>
       </c>
       <c r="D13" s="27" t="s">
-        <v>1179</v>
+        <v>1180</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9166,13 +9169,13 @@
         <v>46311</v>
       </c>
       <c r="B14" s="58" t="s">
-        <v>1180</v>
+        <v>1181</v>
       </c>
       <c r="C14" s="58" t="s">
-        <v>1181</v>
+        <v>1182</v>
       </c>
       <c r="D14" s="58" t="s">
-        <v>1182</v>
+        <v>1183</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9183,10 +9186,10 @@
         <v>58</v>
       </c>
       <c r="C15" s="27" t="s">
-        <v>1183</v>
+        <v>1184</v>
       </c>
       <c r="D15" s="27" t="s">
-        <v>1184</v>
+        <v>1185</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9194,13 +9197,13 @@
         <v>46311</v>
       </c>
       <c r="B16" s="58" t="s">
-        <v>1185</v>
+        <v>1186</v>
       </c>
       <c r="C16" s="58" t="s">
-        <v>1186</v>
+        <v>1187</v>
       </c>
       <c r="D16" s="58" t="s">
-        <v>1187</v>
+        <v>1188</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9211,10 +9214,10 @@
         <v>62</v>
       </c>
       <c r="C17" s="27" t="s">
-        <v>1188</v>
+        <v>1189</v>
       </c>
       <c r="D17" s="27" t="s">
-        <v>1189</v>
+        <v>1190</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9225,10 +9228,10 @@
         <v>436</v>
       </c>
       <c r="C18" s="58" t="s">
-        <v>1190</v>
+        <v>1191</v>
       </c>
       <c r="D18" s="58" t="s">
-        <v>1191</v>
+        <v>1192</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9239,10 +9242,10 @@
         <v>712</v>
       </c>
       <c r="C19" s="27" t="s">
-        <v>1192</v>
+        <v>1193</v>
       </c>
       <c r="D19" s="27" t="s">
-        <v>1193</v>
+        <v>1194</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9250,13 +9253,13 @@
         <v>46311</v>
       </c>
       <c r="B20" s="58" t="s">
-        <v>1194</v>
+        <v>1195</v>
       </c>
       <c r="C20" s="58" t="s">
-        <v>1195</v>
+        <v>1196</v>
       </c>
       <c r="D20" s="58" t="s">
-        <v>1196</v>
+        <v>1197</v>
       </c>
     </row>
   </sheetData>
@@ -10615,7 +10618,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="138" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="138" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A138" s="50" t="s">
         <v>282</v>
       </c>
@@ -10626,7 +10629,7 @@
         <v>283</v>
       </c>
     </row>
-    <row r="139" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="139" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A139" s="42" t="s">
         <v>284</v>
       </c>
@@ -10637,7 +10640,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="140" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="140" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A140" s="50" t="s">
         <v>286</v>
       </c>
@@ -10648,7 +10651,7 @@
         <v>287</v>
       </c>
     </row>
-    <row r="141" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="141" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A141" s="42" t="s">
         <v>288</v>
       </c>
@@ -10659,7 +10662,7 @@
         <v>289</v>
       </c>
     </row>
-    <row r="142" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="142" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A142" s="50" t="s">
         <v>290</v>
       </c>
@@ -10670,7 +10673,7 @@
         <v>291</v>
       </c>
     </row>
-    <row r="143" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="143" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A143" s="42" t="s">
         <v>292</v>
       </c>
@@ -10681,7 +10684,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="144" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="144" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A144" s="50" t="s">
         <v>294</v>
       </c>
@@ -10692,7 +10695,7 @@
         <v>295</v>
       </c>
     </row>
-    <row r="145" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="145" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A145" s="42" t="s">
         <v>296</v>
       </c>
@@ -10703,7 +10706,7 @@
         <v>297</v>
       </c>
     </row>
-    <row r="146" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="146" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A146" s="50" t="s">
         <v>298</v>
       </c>
@@ -10714,7 +10717,7 @@
         <v>299</v>
       </c>
     </row>
-    <row r="147" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="147" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A147" s="42" t="s">
         <v>300</v>
       </c>
@@ -10725,7 +10728,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="148" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="148" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A148" s="50" t="s">
         <v>302</v>
       </c>
@@ -10736,7 +10739,7 @@
         <v>303</v>
       </c>
     </row>
-    <row r="149" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="149" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A149" s="42" t="s">
         <v>304</v>
       </c>
@@ -10747,7 +10750,7 @@
         <v>305</v>
       </c>
     </row>
-    <row r="150" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="150" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A150" s="50" t="s">
         <v>306</v>
       </c>
@@ -10758,7 +10761,7 @@
         <v>307</v>
       </c>
     </row>
-    <row r="151" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="151" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A151" s="42" t="s">
         <v>308</v>
       </c>
@@ -10769,7 +10772,7 @@
         <v>309</v>
       </c>
     </row>
-    <row r="152" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="152" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A152" s="50" t="s">
         <v>310</v>
       </c>
@@ -12961,18 +12964,18 @@
         <v>653</v>
       </c>
       <c r="I6" s="69" t="s">
+        <v>656</v>
+      </c>
+      <c r="J6" s="58" t="s">
         <v>662</v>
-      </c>
-      <c r="J6" s="58" t="s">
-        <v>663</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="27" t="s">
+        <v>663</v>
+      </c>
+      <c r="B7" s="27" t="s">
         <v>664</v>
-      </c>
-      <c r="B7" s="27" t="s">
-        <v>665</v>
       </c>
       <c r="C7" s="27" t="s">
         <v>660</v>
@@ -12996,18 +12999,18 @@
         <v>656</v>
       </c>
       <c r="J7" s="27" t="s">
-        <v>666</v>
+        <v>665</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="58" t="s">
+        <v>666</v>
+      </c>
+      <c r="B8" s="58" t="s">
         <v>667</v>
       </c>
-      <c r="B8" s="58" t="s">
+      <c r="C8" s="58" t="s">
         <v>668</v>
-      </c>
-      <c r="C8" s="58" t="s">
-        <v>669</v>
       </c>
       <c r="D8" s="58" t="s">
         <v>96</v>
@@ -13016,7 +13019,7 @@
         <v>655</v>
       </c>
       <c r="F8" s="58" t="s">
-        <v>669</v>
+        <v>668</v>
       </c>
       <c r="G8" s="43" t="n">
         <v>5</v>
@@ -13025,10 +13028,10 @@
         <v>427</v>
       </c>
       <c r="I8" s="69" t="s">
+        <v>669</v>
+      </c>
+      <c r="J8" s="58" t="s">
         <v>670</v>
-      </c>
-      <c r="J8" s="58" t="s">
-        <v>671</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -13036,10 +13039,10 @@
         <v>406</v>
       </c>
       <c r="B9" s="27" t="s">
+        <v>671</v>
+      </c>
+      <c r="C9" s="27" t="s">
         <v>672</v>
-      </c>
-      <c r="C9" s="27" t="s">
-        <v>673</v>
       </c>
       <c r="D9" s="27" t="s">
         <v>98</v>
@@ -13057,7 +13060,7 @@
         <v>427</v>
       </c>
       <c r="I9" s="69" t="s">
-        <v>656</v>
+        <v>673</v>
       </c>
       <c r="J9" s="27" t="s">
         <v>674</v>
@@ -13089,7 +13092,7 @@
         <v>406</v>
       </c>
       <c r="I10" s="69" t="s">
-        <v>656</v>
+        <v>673</v>
       </c>
       <c r="J10" s="58" t="s">
         <v>677</v>
@@ -13153,7 +13156,7 @@
         <v>545</v>
       </c>
       <c r="I12" s="69" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="J12" s="58" t="s">
         <v>681</v>
@@ -13281,7 +13284,7 @@
         <v>545</v>
       </c>
       <c r="I16" s="69" t="s">
-        <v>656</v>
+        <v>673</v>
       </c>
       <c r="J16" s="58" t="s">
         <v>691</v>
@@ -13313,7 +13316,7 @@
         <v>425</v>
       </c>
       <c r="I17" s="69" t="s">
-        <v>656</v>
+        <v>673</v>
       </c>
       <c r="J17" s="27" t="s">
         <v>694</v>
@@ -13336,7 +13339,7 @@
         <v>655</v>
       </c>
       <c r="F18" s="58" t="s">
-        <v>669</v>
+        <v>668</v>
       </c>
       <c r="G18" s="43" t="n">
         <v>5</v>
@@ -13345,7 +13348,7 @@
         <v>406</v>
       </c>
       <c r="I18" s="69" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="J18" s="58" t="s">
         <v>698</v>
@@ -13359,7 +13362,7 @@
         <v>699</v>
       </c>
       <c r="C19" s="27" t="s">
-        <v>673</v>
+        <v>672</v>
       </c>
       <c r="D19" s="27" t="s">
         <v>98</v>
@@ -13377,7 +13380,7 @@
         <v>406</v>
       </c>
       <c r="I19" s="69" t="s">
-        <v>656</v>
+        <v>673</v>
       </c>
       <c r="J19" s="27" t="s">
         <v>700</v>
@@ -13409,7 +13412,7 @@
         <v>545</v>
       </c>
       <c r="I20" s="69" t="s">
-        <v>656</v>
+        <v>673</v>
       </c>
       <c r="J20" s="58" t="s">
         <v>702</v>
@@ -13441,7 +13444,7 @@
         <v>425</v>
       </c>
       <c r="I21" s="69" t="s">
-        <v>656</v>
+        <v>673</v>
       </c>
       <c r="J21" s="27" t="s">
         <v>706</v>
@@ -13473,7 +13476,7 @@
         <v>689</v>
       </c>
       <c r="I22" s="69" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="J22" s="58" t="s">
         <v>709</v>
@@ -13502,10 +13505,10 @@
         <v>3</v>
       </c>
       <c r="H23" s="27" t="s">
-        <v>667</v>
+        <v>666</v>
       </c>
       <c r="I23" s="69" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="J23" s="27" t="s">
         <v>714</v>
@@ -13537,7 +13540,7 @@
         <v>425</v>
       </c>
       <c r="I24" s="69" t="s">
-        <v>656</v>
+        <v>673</v>
       </c>
       <c r="J24" s="58" t="s">
         <v>715</v>
@@ -13569,7 +13572,7 @@
         <v>438</v>
       </c>
       <c r="I25" s="69" t="s">
-        <v>670</v>
+        <v>673</v>
       </c>
       <c r="J25" s="27" t="s">
         <v>716</v>
@@ -13601,7 +13604,7 @@
         <v>438</v>
       </c>
       <c r="I26" s="69" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="J26" s="58" t="s">
         <v>719</v>
@@ -13633,7 +13636,7 @@
         <v>684</v>
       </c>
       <c r="I27" s="69" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="J27" s="27" t="s">
         <v>720</v>
@@ -13665,7 +13668,7 @@
         <v>684</v>
       </c>
       <c r="I28" s="69" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="J28" s="58" t="s">
         <v>722</v>
@@ -13697,7 +13700,7 @@
         <v>563</v>
       </c>
       <c r="I29" s="69" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="J29" s="27" t="s">
         <v>724</v>
@@ -13711,7 +13714,7 @@
         <v>725</v>
       </c>
       <c r="C30" s="58" t="s">
-        <v>673</v>
+        <v>672</v>
       </c>
       <c r="D30" s="58" t="s">
         <v>100</v>
@@ -13729,7 +13732,7 @@
         <v>563</v>
       </c>
       <c r="I30" s="69" t="s">
-        <v>670</v>
+        <v>673</v>
       </c>
       <c r="J30" s="58" t="s">
         <v>726</v>
@@ -13761,7 +13764,7 @@
         <v>406</v>
       </c>
       <c r="I31" s="69" t="s">
-        <v>656</v>
+        <v>673</v>
       </c>
       <c r="J31" s="27" t="s">
         <v>728</v>
@@ -13784,7 +13787,7 @@
         <v>655</v>
       </c>
       <c r="F32" s="58" t="s">
-        <v>669</v>
+        <v>668</v>
       </c>
       <c r="G32" s="43" t="n">
         <v>8</v>
@@ -13793,7 +13796,7 @@
         <v>599</v>
       </c>
       <c r="I32" s="69" t="s">
-        <v>656</v>
+        <v>673</v>
       </c>
       <c r="J32" s="58" t="s">
         <v>731</v>
@@ -13825,7 +13828,7 @@
         <v>599</v>
       </c>
       <c r="I33" s="69" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="J33" s="27" t="s">
         <v>733</v>
@@ -13857,7 +13860,7 @@
         <v>482</v>
       </c>
       <c r="I34" s="69" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="J34" s="58" t="s">
         <v>737</v>
@@ -13889,7 +13892,7 @@
         <v>734</v>
       </c>
       <c r="I35" s="69" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="J35" s="27" t="s">
         <v>740</v>
@@ -13921,7 +13924,7 @@
         <v>738</v>
       </c>
       <c r="I36" s="69" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="J36" s="58" t="s">
         <v>743</v>
@@ -13953,7 +13956,7 @@
         <v>406</v>
       </c>
       <c r="I37" s="69" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="J37" s="27" t="s">
         <v>747</v>
@@ -13985,7 +13988,7 @@
         <v>744</v>
       </c>
       <c r="I38" s="69" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="J38" s="58" t="s">
         <v>750</v>
@@ -14017,7 +14020,7 @@
         <v>438</v>
       </c>
       <c r="I39" s="69" t="s">
-        <v>656</v>
+        <v>673</v>
       </c>
       <c r="J39" s="27" t="s">
         <v>752</v>
@@ -14049,7 +14052,7 @@
         <v>406</v>
       </c>
       <c r="I40" s="69" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="J40" s="58" t="s">
         <v>753</v>
@@ -14081,7 +14084,7 @@
         <v>482</v>
       </c>
       <c r="I41" s="69" t="s">
-        <v>670</v>
+        <v>673</v>
       </c>
       <c r="J41" s="27" t="s">
         <v>755</v>
@@ -14113,7 +14116,7 @@
         <v>748</v>
       </c>
       <c r="I42" s="69" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="J42" s="58" t="s">
         <v>758</v>
@@ -14145,7 +14148,7 @@
         <v>425</v>
       </c>
       <c r="I43" s="69" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="J43" s="27" t="s">
         <v>762</v>
@@ -14177,7 +14180,7 @@
         <v>425</v>
       </c>
       <c r="I44" s="69" t="s">
-        <v>670</v>
+        <v>673</v>
       </c>
       <c r="J44" s="58" t="s">
         <v>765</v>
@@ -14209,7 +14212,7 @@
         <v>695</v>
       </c>
       <c r="I45" s="69" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="J45" s="27" t="s">
         <v>768</v>
@@ -14241,7 +14244,7 @@
         <v>689</v>
       </c>
       <c r="I46" s="69" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="J46" s="58" t="s">
         <v>771</v>
@@ -14273,7 +14276,7 @@
         <v>406</v>
       </c>
       <c r="I47" s="69" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="J47" s="27" t="s">
         <v>774</v>
@@ -14305,7 +14308,7 @@
         <v>738</v>
       </c>
       <c r="I48" s="69" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="J48" s="58" t="s">
         <v>777</v>
@@ -14337,7 +14340,7 @@
         <v>766</v>
       </c>
       <c r="I49" s="69" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="J49" s="27" t="s">
         <v>781</v>
@@ -14369,7 +14372,7 @@
         <v>703</v>
       </c>
       <c r="I50" s="69" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="J50" s="58" t="s">
         <v>785</v>
@@ -14401,7 +14404,7 @@
         <v>717</v>
       </c>
       <c r="I51" s="69" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="J51" s="27" t="s">
         <v>789</v>
@@ -14433,7 +14436,7 @@
         <v>608</v>
       </c>
       <c r="I52" s="69" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="J52" s="58" t="s">
         <v>792</v>
@@ -14465,7 +14468,7 @@
         <v>790</v>
       </c>
       <c r="I53" s="69" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="J53" s="27" t="s">
         <v>794</v>
@@ -14497,7 +14500,7 @@
         <v>717</v>
       </c>
       <c r="I54" s="69" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="J54" s="58" t="s">
         <v>797</v>
@@ -14529,7 +14532,7 @@
         <v>741</v>
       </c>
       <c r="I55" s="69" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="J55" s="27" t="s">
         <v>801</v>
@@ -14561,7 +14564,7 @@
         <v>563</v>
       </c>
       <c r="I56" s="69" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="J56" s="58" t="s">
         <v>804</v>
@@ -14593,7 +14596,7 @@
         <v>786</v>
       </c>
       <c r="I57" s="69" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="J57" s="27" t="s">
         <v>807</v>
@@ -14625,7 +14628,7 @@
         <v>689</v>
       </c>
       <c r="I58" s="69" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="J58" s="58" t="s">
         <v>810</v>
@@ -14639,7 +14642,7 @@
         <v>812</v>
       </c>
       <c r="C59" s="27" t="s">
-        <v>673</v>
+        <v>672</v>
       </c>
       <c r="D59" s="27" t="s">
         <v>102</v>
@@ -14657,7 +14660,7 @@
         <v>703</v>
       </c>
       <c r="I59" s="69" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="J59" s="27" t="s">
         <v>813</v>
@@ -14689,7 +14692,7 @@
         <v>805</v>
       </c>
       <c r="I60" s="69" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="J60" s="58" t="s">
         <v>817</v>
@@ -14721,7 +14724,7 @@
         <v>805</v>
       </c>
       <c r="I61" s="69" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="J61" s="27" t="s">
         <v>820</v>
@@ -14753,7 +14756,7 @@
         <v>689</v>
       </c>
       <c r="I62" s="69" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="J62" s="58" t="s">
         <v>823</v>
@@ -14785,7 +14788,7 @@
         <v>805</v>
       </c>
       <c r="I63" s="69" t="s">
-        <v>656</v>
+        <v>673</v>
       </c>
       <c r="J63" s="27" t="s">
         <v>827</v>
@@ -14817,7 +14820,7 @@
         <v>818</v>
       </c>
       <c r="I64" s="69" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="J64" s="58" t="s">
         <v>830</v>
@@ -14849,7 +14852,7 @@
         <v>805</v>
       </c>
       <c r="I65" s="69" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="J65" s="27" t="s">
         <v>833</v>
@@ -14881,7 +14884,7 @@
         <v>763</v>
       </c>
       <c r="I66" s="69" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="J66" s="58" t="s">
         <v>836</v>
@@ -14913,7 +14916,7 @@
         <v>818</v>
       </c>
       <c r="I67" s="69" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="J67" s="27" t="s">
         <v>839</v>
@@ -14945,7 +14948,7 @@
         <v>837</v>
       </c>
       <c r="I68" s="69" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="J68" s="58" t="s">
         <v>842</v>
@@ -14977,7 +14980,7 @@
         <v>831</v>
       </c>
       <c r="I69" s="69" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="J69" s="27" t="s">
         <v>845</v>
@@ -15156,7 +15159,7 @@
       <c r="F85" s="73"/>
       <c r="G85" s="32" t="n">
         <f aca="false">SUMIF(I$5:I$80,"Done",G$5:G$80)</f>
-        <v>8</v>
+        <v>52</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -15167,7 +15170,7 @@
       <c r="F86" s="73"/>
       <c r="G86" s="74" t="n">
         <f aca="false">IF(G83=0,0,SUMIFS(G$5:G$80,E$5:E$80,"Must",I$5:I$80,"Done")/G83)</f>
-        <v>0.0261437908496732</v>
+        <v>0.169934640522876</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -15248,7 +15251,7 @@
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A93" s="75" t="s">
-        <v>669</v>
+        <v>668</v>
       </c>
       <c r="B93" s="75"/>
       <c r="C93" s="32" t="n">

</xml_diff>

<commit_message>
Pause and options menu (F51); plan: F19-F21 and F53 done, F51 in progress
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018inbrQHz2eFfbj9ny1keZA
</commit_message>
<xml_diff>
--- a/docs/Vinland_Game_Development_Plan.xlsx
+++ b/docs/Vinland_Game_Development_Plan.xlsx
@@ -86,7 +86,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1973" uniqueCount="1247">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1976" uniqueCount="1249">
   <si>
     <t xml:space="preserve">VINLAND</t>
   </si>
@@ -2446,7 +2446,7 @@
     <t xml:space="preserve">Trade</t>
   </si>
   <si>
-    <t xml:space="preserve">Trade raises goodwill; weapon sale, killing, palisade, loose bull raise fear toward the cap.  [Fear clock started: far hunting raises fear (cap 5). Goodwill and the market still to come.]</t>
+    <t xml:space="preserve">Trade raises goodwill; weapon sale, killing, palisade, loose bull raise fear toward the cap.  [Built: goodwill 0-10 from trades (+2 for a generous one), fear 0-5 from far hunting, the bull and weapon sales; fear eases 0.5 a quiet week; at the cap trade stops and raids take animals or hurt a crew member.]</t>
   </si>
   <si>
     <t xml:space="preserve">F20</t>
@@ -2455,7 +2455,7 @@
     <t xml:space="preserve">Market day</t>
   </si>
   <si>
-    <t xml:space="preserve">Milk and red cloth trade; visitors have wants of their own and leave when fear rises.</t>
+    <t xml:space="preserve">Milk and red cloth trade; visitors have wants of their own and leave when fear rises.  [Built: visitors come on about 6% of summer days (more with goodwill), bring 3-8 pelts; offer red cloth and milk on a trade screen; goodwill lowers the price; sending them away costs goodwill; auto-resolved in week mode. Visitors are neutral placeholders pending F59.]</t>
   </si>
   <si>
     <t xml:space="preserve">F21</t>
@@ -2464,7 +2464,7 @@
     <t xml:space="preserve">Bull and weapon-sale events</t>
   </si>
   <si>
-    <t xml:space="preserve">Either event can break the market; neither is a cutscene.</t>
+    <t xml:space="preserve">Either event can break the market; neither is a cutscene.  [Built: an unpenned bull breaks loose 1 in 4 markets until the byre is up (fear +2, market ends); penning keeps one crew member back. At goodwill 2+ they may ask for iron: refusing costs 0.5 goodwill, selling two blades gives 6 pelts and fear +2.]</t>
   </si>
   <si>
     <t xml:space="preserve">F22</t>
@@ -2539,7 +2539,7 @@
     <t xml:space="preserve">Main menu, options, pause</t>
   </si>
   <si>
-    <t xml:space="preserve">Options cover remaps, haptic strength, text size, and ironman.</t>
+    <t xml:space="preserve">Options cover remaps, haptic strength, text size, and ironman.  [Built: pause menu on Back / P with resume, difficulty, vibration on/off, prompts auto/always/never, save and quit to title; settings persist in user://settings.json. Still to do: remaps, haptic strength, text size, ironman.]</t>
   </si>
   <si>
     <t xml:space="preserve">F52</t>
@@ -2557,7 +2557,7 @@
     <t xml:space="preserve">Eriksfjord loadout</t>
   </si>
   <si>
-    <t xml:space="preserve">Player picks people, animals, and goods against the hull before leaving.</t>
+    <t xml:space="preserve">Player picks people, animals, and goods against the hull before leaving.  [Built: Eriksfjord loadout screen: people, cattle, sheep, food, drink, fodder, red cloth, iron against the 24-unit hull with days-of-stores readouts and warnings; Y restores the HoldCheck load; an overloaded hull will not sail; cloth and iron carry into the camp market.]</t>
   </si>
   <si>
     <t xml:space="preserve">F59</t>
@@ -3827,6 +3827,12 @@
   </si>
   <si>
     <t xml:space="preserve">One page now shows scope load, hold math, revenue, risk, and gate status.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F19, F20, F21, F53 marked Done; F51 In progress with the pause and options menu built.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Market at the shore, the Eriksfjord loadout and the pause menu are in the build with tests.</t>
   </si>
 </sst>
 </file>
@@ -5031,11 +5037,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="34176278"/>
-        <c:axId val="17074735"/>
+        <c:axId val="47226815"/>
+        <c:axId val="18458890"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="34176278"/>
+        <c:axId val="47226815"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5067,7 +5073,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="17074735"/>
+        <c:crossAx val="18458890"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -5075,7 +5081,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="17074735"/>
+        <c:axId val="18458890"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5151,7 +5157,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="34176278"/>
+        <c:crossAx val="47226815"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -5190,9 +5196,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>741960</xdr:colOff>
+      <xdr:colOff>741600</xdr:colOff>
       <xdr:row>40</xdr:row>
-      <xdr:rowOff>58320</xdr:rowOff>
+      <xdr:rowOff>57960</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -5201,7 +5207,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="0" y="6562800"/>
-        <a:ext cx="5393880" cy="2153880"/>
+        <a:ext cx="5393520" cy="2153520"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -6116,7 +6122,7 @@
       </c>
       <c r="B55" s="5" t="str">
         <f aca="false">COUNTIF(Backlog!I5:I80,"Done")&amp;" of "&amp;COUNTA(Backlog!A5:A80)</f>
-        <v>7 of 65</v>
+        <v>11 of 65</v>
       </c>
       <c r="C55" s="31" t="s">
         <v>68</v>
@@ -6138,7 +6144,7 @@
       </c>
       <c r="B56" s="38" t="n">
         <f aca="false">Backlog!G86</f>
-        <v>0.169934640522876</v>
+        <v>0.23202614379085</v>
       </c>
       <c r="C56" s="34" t="s">
         <v>71</v>
@@ -9146,7 +9152,7 @@
     <tabColor rgb="FFC4A46A"/>
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:D20"/>
+  <dimension ref="A1:D21"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="14"/>
@@ -9407,6 +9413,20 @@
       </c>
       <c r="D20" s="58" t="s">
         <v>1246</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="102" t="n">
+        <v>46313</v>
+      </c>
+      <c r="B21" s="58" t="s">
+        <v>451</v>
+      </c>
+      <c r="C21" s="58" t="s">
+        <v>1247</v>
+      </c>
+      <c r="D21" s="58" t="s">
+        <v>1248</v>
       </c>
     </row>
   </sheetData>
@@ -10996,14 +11016,14 @@
         <v>323</v>
       </c>
     </row>
-    <row r="160" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="160" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A160" s="24" t="s">
         <v>324</v>
       </c>
       <c r="B160" s="24"/>
       <c r="C160" s="24"/>
     </row>
-    <row r="161" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="161" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A161" s="9" t="s">
         <v>132</v>
       </c>
@@ -11014,7 +11034,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="162" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="162" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A162" s="42" t="s">
         <v>325</v>
       </c>
@@ -11025,7 +11045,7 @@
         <v>326</v>
       </c>
     </row>
-    <row r="163" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="163" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A163" s="50" t="s">
         <v>327</v>
       </c>
@@ -11036,7 +11056,7 @@
         <v>328</v>
       </c>
     </row>
-    <row r="164" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="164" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A164" s="42" t="s">
         <v>329</v>
       </c>
@@ -11047,7 +11067,7 @@
         <v>330</v>
       </c>
     </row>
-    <row r="165" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="165" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A165" s="50" t="s">
         <v>331</v>
       </c>
@@ -11058,7 +11078,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="166" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="166" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A166" s="42" t="s">
         <v>333</v>
       </c>
@@ -11069,7 +11089,7 @@
         <v>335</v>
       </c>
     </row>
-    <row r="167" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="167" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A167" s="50" t="s">
         <v>336</v>
       </c>
@@ -11080,7 +11100,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="168" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="168" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A168" s="42" t="s">
         <v>338</v>
       </c>
@@ -11091,7 +11111,7 @@
         <v>339</v>
       </c>
     </row>
-    <row r="169" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="169" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A169" s="50" t="s">
         <v>340</v>
       </c>
@@ -11102,7 +11122,7 @@
         <v>341</v>
       </c>
     </row>
-    <row r="170" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="170" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A170" s="42" t="s">
         <v>342</v>
       </c>
@@ -11113,7 +11133,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="171" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="171" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A171" s="50" t="s">
         <v>344</v>
       </c>
@@ -11124,7 +11144,7 @@
         <v>345</v>
       </c>
     </row>
-    <row r="172" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="172" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A172" s="42" t="s">
         <v>346</v>
       </c>
@@ -11135,7 +11155,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="173" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="173" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A173" s="50" t="s">
         <v>348</v>
       </c>
@@ -11146,7 +11166,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="174" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="174" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A174" s="42" t="s">
         <v>350</v>
       </c>
@@ -11157,7 +11177,7 @@
         <v>351</v>
       </c>
     </row>
-    <row r="175" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="175" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A175" s="50" t="s">
         <v>352</v>
       </c>
@@ -11168,7 +11188,7 @@
         <v>353</v>
       </c>
     </row>
-    <row r="176" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="176" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A176" s="42" t="s">
         <v>354</v>
       </c>
@@ -11179,7 +11199,7 @@
         <v>355</v>
       </c>
     </row>
-    <row r="177" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="177" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A177" s="50" t="s">
         <v>356</v>
       </c>
@@ -11190,7 +11210,7 @@
         <v>357</v>
       </c>
     </row>
-    <row r="178" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="178" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A178" s="42" t="s">
         <v>358</v>
       </c>
@@ -11201,7 +11221,7 @@
         <v>359</v>
       </c>
     </row>
-    <row r="179" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="179" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A179" s="50" t="s">
         <v>360</v>
       </c>
@@ -14290,7 +14310,7 @@
         <v>531</v>
       </c>
       <c r="I34" s="69" t="s">
-        <v>722</v>
+        <v>705</v>
       </c>
       <c r="J34" s="58" t="s">
         <v>786</v>
@@ -14322,7 +14342,7 @@
         <v>783</v>
       </c>
       <c r="I35" s="69" t="s">
-        <v>718</v>
+        <v>705</v>
       </c>
       <c r="J35" s="27" t="s">
         <v>789</v>
@@ -14354,7 +14374,7 @@
         <v>787</v>
       </c>
       <c r="I36" s="69" t="s">
-        <v>718</v>
+        <v>705</v>
       </c>
       <c r="J36" s="58" t="s">
         <v>792</v>
@@ -14642,7 +14662,7 @@
         <v>744</v>
       </c>
       <c r="I45" s="69" t="s">
-        <v>718</v>
+        <v>722</v>
       </c>
       <c r="J45" s="27" t="s">
         <v>817</v>
@@ -14706,7 +14726,7 @@
         <v>455</v>
       </c>
       <c r="I47" s="69" t="s">
-        <v>718</v>
+        <v>705</v>
       </c>
       <c r="J47" s="27" t="s">
         <v>823</v>
@@ -15589,7 +15609,7 @@
       <c r="F85" s="73"/>
       <c r="G85" s="32" t="n">
         <f aca="false">SUMIF(I$5:I$80,"Done",G$5:G$80)</f>
-        <v>52</v>
+        <v>71</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -15600,7 +15620,7 @@
       <c r="F86" s="73"/>
       <c r="G86" s="74" t="n">
         <f aca="false">IF(G83=0,0,SUMIFS(G$5:G$80,E$5:E$80,"Must",I$5:I$80,"Done")/G83)</f>
-        <v>0.169934640522876</v>
+        <v>0.23202614379085</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Plan: F04, F14, F15 progress; work mini-game payoff knobs
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018inbrQHz2eFfbj9ny1keZA
</commit_message>
<xml_diff>
--- a/docs/Vinland_Game_Development_Plan.xlsx
+++ b/docs/Vinland_Game_Development_Plan.xlsx
@@ -86,7 +86,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1997" uniqueCount="1267">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2000" uniqueCount="1270">
   <si>
     <t xml:space="preserve">VINLAND</t>
   </si>
@@ -2332,7 +2332,7 @@
     <t xml:space="preserve">Sun board mini-game</t>
   </si>
   <si>
-    <t xml:space="preserve">Overcast skips it; a snatched shadow keeps yesterday's error.</t>
+    <t xml:space="preserve">Overcast skips it; a snatched shadow keeps yesterday's error.  [Playable: noon sun board on sunny days (fair, calm, drift ice; a gap in low cloud 35%); turn the disk, set the peg, steady through the roll, take the reading; a snatched shadow is partial. The day uses the better of sun and stars. Novice keyboard/pad 100/100% Forgiving, 100/96% Standard, 42/79% Hard.]</t>
   </si>
   <si>
     <t xml:space="preserve">Hand-line fishing</t>
@@ -2461,13 +2461,13 @@
     <t xml:space="preserve">Net throw</t>
   </si>
   <si>
-    <t xml:space="preserve">An empty throw spends the day.</t>
+    <t xml:space="preserve">An empty throw spends the day.  [Playable in the camp (B on the Fish row): aim ahead of the school, cast, close with both triggers at the school depth; deeper in rain, hidden in fog until near; one throw a day (two on Forgiving), up to 48 person-days. Novice 96/100% Forgiving, 71/92% Standard.]</t>
   </si>
   <si>
     <t xml:space="preserve">Drying and smoke rack</t>
   </si>
   <si>
-    <t xml:space="preserve">Two fair days turn fresh fish into a food unit.  [Smoke-and-dry job turns surplus fresh fish into stores on fair days (90% kept). Rack mini-game (MG9) still to come.]</t>
+    <t xml:space="preserve">Two fair days turn fresh fish into a food unit.  [Smoke-and-dry job turns surplus fresh fish into stores on fair days (90% kept). Rack fire mini-game (MG9) built: steer the smoke under the rack through gusts, hold the heat in the band; your fire cures up to 1.5x a dryer at 60-100% yield, a case-hardened rack loses your share.]</t>
   </si>
   <si>
     <t xml:space="preserve">Livestock, milk, hay</t>
@@ -3887,6 +3887,15 @@
   </si>
   <si>
     <t xml:space="preserve">Market at the shore, the Eriksfjord loadout and the pause menu are in the build with tests.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Backlog, Assumptions</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F04 sun board, F14 net and the MG9 smoke rack built; new WORK MINI-GAME PAYOFFS knobs on Assumptions.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The sun board, net and smoke rack are playable, tested with expert bots and novice models, and tuned per difficulty.</t>
   </si>
 </sst>
 </file>
@@ -5095,11 +5104,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="81071095"/>
-        <c:axId val="38110597"/>
+        <c:axId val="79622641"/>
+        <c:axId val="37277396"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="81071095"/>
+        <c:axId val="79622641"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5131,7 +5140,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="38110597"/>
+        <c:crossAx val="37277396"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -5139,7 +5148,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="38110597"/>
+        <c:axId val="37277396"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5215,7 +5224,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="81071095"/>
+        <c:crossAx val="79622641"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -5254,9 +5263,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>741240</xdr:colOff>
+      <xdr:colOff>740520</xdr:colOff>
       <xdr:row>40</xdr:row>
-      <xdr:rowOff>57600</xdr:rowOff>
+      <xdr:rowOff>56880</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -5265,7 +5274,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="0" y="6562800"/>
-        <a:ext cx="5393160" cy="2153160"/>
+        <a:ext cx="5392440" cy="2152440"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -9210,7 +9219,7 @@
     <tabColor rgb="FFC4A46A"/>
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:D21"/>
+  <dimension ref="A1:D22"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="14"/>
@@ -9485,6 +9494,20 @@
       </c>
       <c r="D21" s="59" t="s">
         <v>1266</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="103" t="n">
+        <v>46313</v>
+      </c>
+      <c r="B22" s="59" t="s">
+        <v>1267</v>
+      </c>
+      <c r="C22" s="59" t="s">
+        <v>1268</v>
+      </c>
+      <c r="D22" s="59" t="s">
+        <v>1269</v>
       </c>
     </row>
   </sheetData>
@@ -13768,7 +13791,7 @@
         <v>612</v>
       </c>
       <c r="I12" s="70" t="s">
-        <v>736</v>
+        <v>740</v>
       </c>
       <c r="J12" s="59" t="s">
         <v>748</v>
@@ -14312,7 +14335,7 @@
         <v>630</v>
       </c>
       <c r="I29" s="70" t="s">
-        <v>736</v>
+        <v>740</v>
       </c>
       <c r="J29" s="27" t="s">
         <v>791</v>

</xml_diff>